<commit_message>
Update MLB weather 2026-07-16 12:29 AM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -206,10 +206,10 @@
     <t>OPEN-AIR PARK</t>
   </si>
   <si>
-    <t>Partly cloudy</t>
-  </si>
-  <si>
-    <t>🟢 5.0 mph Out to RF</t>
+    <t>Mostly clear</t>
+  </si>
+  <si>
+    <t>🔴 5.1 mph In from LF</t>
   </si>
   <si>
     <t>W</t>
@@ -221,19 +221,22 @@
     <t>B</t>
   </si>
   <si>
-    <t>Density 86 | Wind 44 | Temp 70 | Altitude 66 | Confidence 90%</t>
+    <t>Density 86 | Wind 44 | Temp 71 | Altitude 66 | Confidence 90%</t>
   </si>
   <si>
     <t>🟨 Neutral</t>
   </si>
   <si>
-    <t>FIRST RUN</t>
+    <t>IMPROVING</t>
+  </si>
+  <si>
+    <t>MODERATE</t>
   </si>
   <si>
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-15 09:24:18 PM PDT</t>
+    <t>2026-07-16 12:29:18 AM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,10 +470,10 @@
     <t>10:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-16 04:24:18 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-16T04:13:22+00:00</t>
+    <t>2026-07-16 07:29:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-16T06:30:59+00:00</t>
   </si>
   <si>
     <t>YES</t>
@@ -489,9 +492,6 @@
   </si>
   <si>
     <t>2026-07-16T23:00</t>
-  </si>
-  <si>
-    <t>Mostly clear</t>
   </si>
   <si>
     <t>WNW</t>
@@ -961,7 +961,7 @@
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="27.7109375" customWidth="1"/>
     <col min="12" max="12" width="33.7109375" customWidth="1"/>
-    <col min="13" max="13" width="21.7109375" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" customWidth="1"/>
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" customWidth="1"/>
@@ -1186,34 +1186,34 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>94.3</v>
+        <v>94.5</v>
       </c>
       <c r="L2">
-        <v>42.3</v>
+        <v>42</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>-4.9</v>
+        <v>-5.1</v>
       </c>
       <c r="Q2">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="R2">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
       </c>
       <c r="U2">
-        <v>14.4</v>
+        <v>23.2</v>
       </c>
       <c r="V2">
         <v>59.1</v>
@@ -1234,7 +1234,7 @@
         <v>2.7</v>
       </c>
       <c r="AB2">
-        <v>89.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
@@ -1252,16 +1252,16 @@
         <v>90</v>
       </c>
       <c r="AH2">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="AI2">
         <v>1.2</v>
       </c>
       <c r="AJ2">
-        <v>1.1387</v>
+        <v>1.1385</v>
       </c>
       <c r="AK2">
-        <v>2296</v>
+        <v>2305</v>
       </c>
       <c r="AL2">
         <v>1008.8</v>
@@ -1270,16 +1270,16 @@
         <v>64.8</v>
       </c>
       <c r="AN2">
-        <v>91.5</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="AO2">
-        <v>43.7</v>
+        <v>43.6</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1291,19 +1291,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>18.3</v>
+        <v>24</v>
       </c>
       <c r="AV2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AW2">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="AX2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AY2">
-        <v>10.9</v>
+        <v>58.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1371,7 +1371,7 @@
     <col min="28" max="28" width="27.7109375" customWidth="1"/>
     <col min="29" max="29" width="17.7109375" customWidth="1"/>
     <col min="30" max="30" width="25.7109375" customWidth="1"/>
-    <col min="31" max="31" width="15.7109375" customWidth="1"/>
+    <col min="31" max="31" width="14.7109375" customWidth="1"/>
     <col min="32" max="32" width="10.7109375" customWidth="1"/>
     <col min="33" max="33" width="14.7109375" customWidth="1"/>
     <col min="34" max="34" width="13.7109375" customWidth="1"/>
@@ -1426,211 +1426,211 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="BV1" s="1" t="s">
         <v>48</v>
@@ -1639,16 +1639,16 @@
         <v>47</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="BY1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="BZ1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="CA1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:79">
@@ -1665,40 +1665,40 @@
         <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F2" t="s">
         <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J2">
-        <v>10.9</v>
+        <v>58.3</v>
       </c>
       <c r="K2">
-        <v>18.8</v>
+        <v>15.7</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>2.06</v>
+        <v>2.44</v>
       </c>
       <c r="N2">
-        <v>2.6</v>
+        <v>3.01</v>
       </c>
       <c r="O2">
-        <v>4.61</v>
+        <v>5.12</v>
       </c>
       <c r="P2">
-        <v>9.9</v>
+        <v>9.5</v>
       </c>
       <c r="Q2">
         <v>1.1</v>
@@ -1710,25 +1710,25 @@
         <v>75</v>
       </c>
       <c r="T2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="U2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="V2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="W2">
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>17.7</v>
+        <v>20.6</v>
       </c>
       <c r="Y2">
-        <v>89.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="Z2">
-        <v>67.90000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1746,73 +1746,73 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>94.3</v>
+        <v>94.5</v>
       </c>
       <c r="AG2">
-        <v>96.2</v>
+        <v>96.5</v>
       </c>
       <c r="AH2">
         <v>66.59999999999999</v>
       </c>
       <c r="AI2">
-        <v>42.3</v>
+        <v>42</v>
       </c>
       <c r="AJ2">
-        <v>1008.1</v>
+        <v>1007.9</v>
       </c>
       <c r="AK2">
-        <v>1010.3</v>
+        <v>1010.2</v>
       </c>
       <c r="AL2">
-        <v>71.3</v>
+        <v>36.6</v>
       </c>
       <c r="AM2">
-        <v>14.4</v>
+        <v>23.2</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>31.4</v>
+        <v>35.1</v>
       </c>
       <c r="AP2">
-        <v>1038</v>
+        <v>1122</v>
       </c>
       <c r="AQ2">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AR2">
-        <v>20</v>
+        <v>20.6</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>280.5</v>
+        <v>281.1</v>
       </c>
       <c r="AU2">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="AV2">
-        <v>-5.5</v>
+        <v>-5.7</v>
       </c>
       <c r="AW2">
         <v>5.4</v>
       </c>
       <c r="AX2">
+        <v>-0.2</v>
+      </c>
+      <c r="AY2">
+        <v>-5.1</v>
+      </c>
+      <c r="AZ2">
+        <v>5.1</v>
+      </c>
+      <c r="BA2">
+        <v>9.5</v>
+      </c>
+      <c r="BB2">
         <v>-0.1</v>
-      </c>
-      <c r="AY2">
-        <v>-4.9</v>
-      </c>
-      <c r="AZ2">
-        <v>5</v>
-      </c>
-      <c r="BA2">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="BB2">
-        <v>-0</v>
       </c>
       <c r="BC2">
         <v>0.9</v>
@@ -1830,13 +1830,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1316</v>
+        <v>1.131</v>
       </c>
       <c r="BI2" t="s">
         <v>159</v>
       </c>
       <c r="BJ2">
-        <v>2503</v>
+        <v>2524</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1845,49 +1845,49 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>70</v>
+        <v>70.2</v>
       </c>
       <c r="BN2">
         <v>1.048</v>
       </c>
       <c r="BO2">
-        <v>74.5</v>
+        <v>74.8</v>
       </c>
       <c r="BP2">
-        <v>65.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="BQ2">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="BR2">
         <v>56.3</v>
       </c>
       <c r="BS2">
-        <v>42.9</v>
+        <v>42.2</v>
       </c>
       <c r="BT2">
-        <v>18.3</v>
+        <v>24</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="BW2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BX2">
         <v>93</v>
       </c>
       <c r="BY2">
-        <v>94</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="BZ2">
         <v>10</v>
       </c>
       <c r="CA2">
-        <v>9.4</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1904,25 +1904,25 @@
         <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J3">
-        <v>10.9</v>
+        <v>58.3</v>
       </c>
       <c r="K3">
-        <v>19.8</v>
+        <v>16.7</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -1934,7 +1934,7 @@
         <v>2.86</v>
       </c>
       <c r="O3">
-        <v>4.16</v>
+        <v>4.98</v>
       </c>
       <c r="P3">
         <v>13</v>
@@ -1949,19 +1949,19 @@
         <v>100</v>
       </c>
       <c r="T3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="U3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="V3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="W3">
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>16.5</v>
+        <v>16.8</v>
       </c>
       <c r="Y3">
         <v>89.09999999999999</v>
@@ -1982,7 +1982,7 @@
         <v>1.6</v>
       </c>
       <c r="AE3" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="AF3">
         <v>91.8</v>
@@ -2006,7 +2006,7 @@
         <v>40</v>
       </c>
       <c r="AM3">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AN3">
         <v>0</v>
@@ -2105,16 +2105,16 @@
         <v>46.9</v>
       </c>
       <c r="BT3">
-        <v>12.4</v>
+        <v>14.6</v>
       </c>
       <c r="BU3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BV3">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="BW3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BX3">
         <v>91</v>
@@ -2143,25 +2143,25 @@
         <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J4">
-        <v>10.9</v>
+        <v>58.3</v>
       </c>
       <c r="K4">
-        <v>20.8</v>
+        <v>17.7</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -2173,7 +2173,7 @@
         <v>2.23</v>
       </c>
       <c r="O4">
-        <v>2.96</v>
+        <v>3.61</v>
       </c>
       <c r="P4">
         <v>12.1</v>
@@ -2188,22 +2188,22 @@
         <v>100</v>
       </c>
       <c r="T4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="U4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="V4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="W4">
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="Y4">
-        <v>90.90000000000001</v>
+        <v>91</v>
       </c>
       <c r="Z4">
         <v>51.1</v>
@@ -2221,7 +2221,7 @@
         <v>1.6</v>
       </c>
       <c r="AE4" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="AF4">
         <v>88.59999999999999</v>
@@ -2245,7 +2245,7 @@
         <v>39.5</v>
       </c>
       <c r="AM4">
-        <v>8.800000000000001</v>
+        <v>16</v>
       </c>
       <c r="AN4">
         <v>0</v>
@@ -2344,16 +2344,16 @@
         <v>51.6</v>
       </c>
       <c r="BT4">
-        <v>6.4</v>
+        <v>10.3</v>
       </c>
       <c r="BU4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BV4">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="BW4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BX4">
         <v>88</v>
@@ -2382,25 +2382,25 @@
         <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J5">
-        <v>10.9</v>
+        <v>58.3</v>
       </c>
       <c r="K5">
-        <v>21.8</v>
+        <v>18.7</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -2412,7 +2412,7 @@
         <v>1.16</v>
       </c>
       <c r="O5">
-        <v>1.6</v>
+        <v>1.95</v>
       </c>
       <c r="P5">
         <v>13.3</v>
@@ -2427,22 +2427,22 @@
         <v>100</v>
       </c>
       <c r="T5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="U5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="V5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="W5">
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="Y5">
-        <v>92.3</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="Z5">
         <v>46.4</v>
@@ -2460,7 +2460,7 @@
         <v>1.6</v>
       </c>
       <c r="AE5" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="AF5">
         <v>85.7</v>
@@ -2484,7 +2484,7 @@
         <v>40.5</v>
       </c>
       <c r="AM5">
-        <v>2.5</v>
+        <v>12.8</v>
       </c>
       <c r="AN5">
         <v>0</v>
@@ -2583,16 +2583,16 @@
         <v>55</v>
       </c>
       <c r="BT5">
-        <v>1.7</v>
+        <v>7.4</v>
       </c>
       <c r="BU5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BV5">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="BW5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BX5">
         <v>86</v>
@@ -2712,7 +2712,7 @@
         <v>65</v>
       </c>
       <c r="G2">
-        <v>89.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="H2">
         <v>6</v>
@@ -2730,10 +2730,10 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>91.5</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="N2">
-        <v>2296</v>
+        <v>2305</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 12:30 AM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -236,7 +236,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 12:29:18 AM PDT</t>
+    <t>2026-07-16 12:30:07 AM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -470,7 +470,7 @@
     <t>10:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-16 07:29:18 UTC</t>
+    <t>2026-07-16 07:30:07 UTC</t>
   </si>
   <si>
     <t>2026-07-16T06:30:59+00:00</t>
@@ -1303,7 +1303,7 @@
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1680,7 +1680,7 @@
         <v>150</v>
       </c>
       <c r="J2">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="K2">
         <v>15.7</v>
@@ -1872,7 +1872,7 @@
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="BW2" t="s">
         <v>70</v>
@@ -1919,7 +1919,7 @@
         <v>150</v>
       </c>
       <c r="J3">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="K3">
         <v>16.7</v>
@@ -2158,7 +2158,7 @@
         <v>150</v>
       </c>
       <c r="J4">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="K4">
         <v>17.7</v>
@@ -2397,7 +2397,7 @@
         <v>150</v>
       </c>
       <c r="J5">
-        <v>58.3</v>
+        <v>59.1</v>
       </c>
       <c r="K5">
         <v>18.7</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 01:24 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -191,294 +191,297 @@
     <t>New York Mets @ Philadelphia Phillies</t>
   </si>
   <si>
-    <t>04:10 PM</t>
+    <t>03:10 PM</t>
+  </si>
+  <si>
+    <t>06:10 PM EDT</t>
+  </si>
+  <si>
+    <t>Citizens Bank Park</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>OPEN-AIR PARK</t>
+  </si>
+  <si>
+    <t>Clear</t>
+  </si>
+  <si>
+    <t>🟢 7.2 mph Out to RF</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>FORECAST MODEL</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>Density 88 | Wind 48 | Temp 72 | Altitude 67 | Confidence 88%</t>
+  </si>
+  <si>
+    <t>🟢 Good</t>
+  </si>
+  <si>
+    <t>IMPROVING RAPIDLY</t>
+  </si>
+  <si>
+    <t>MODERATE</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>2026-07-16 01:24:56 PM PDT</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Target Local</t>
+  </si>
+  <si>
+    <t>Forecast Run UTC</t>
+  </si>
+  <si>
+    <t>NWS Forecast Updated</t>
+  </si>
+  <si>
+    <t>Hours Until Game</t>
+  </si>
+  <si>
+    <t>Temperature Model Spread F</t>
+  </si>
+  <si>
+    <t>Wind Model Spread MPH</t>
+  </si>
+  <si>
+    <t>Precip Model Spread Pct</t>
+  </si>
+  <si>
+    <t>Wind Direction Spread Degrees</t>
+  </si>
+  <si>
+    <t>Wind Toward CF Spread MPH</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing Out %</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing In %</t>
+  </si>
+  <si>
+    <t>Exact-Time Interpolation</t>
+  </si>
+  <si>
+    <t>Interpolation Lower Time</t>
+  </si>
+  <si>
+    <t>Interpolation Upper Time</t>
+  </si>
+  <si>
+    <t>Interpolation Fraction</t>
+  </si>
+  <si>
+    <t>Ensemble Disagreement Score</t>
+  </si>
+  <si>
+    <t>Weather Confidence %</t>
+  </si>
+  <si>
+    <t>Confidence-Adjusted HR Score</t>
+  </si>
+  <si>
+    <t>Park Wind Exposure</t>
+  </si>
+  <si>
+    <t>Park Temperature Offset F</t>
+  </si>
+  <si>
+    <t>Park Carry Bias</t>
+  </si>
+  <si>
+    <t>Microclimate Adjustment</t>
+  </si>
+  <si>
+    <t>Conditions</t>
+  </si>
+  <si>
+    <t>Temp F</t>
+  </si>
+  <si>
+    <t>Feels Like F</t>
+  </si>
+  <si>
+    <t>Dew Point F</t>
+  </si>
+  <si>
+    <t>RH %</t>
+  </si>
+  <si>
+    <t>Surface Pressure hPa</t>
+  </si>
+  <si>
+    <t>Sea Level Pressure hPa</t>
+  </si>
+  <si>
+    <t>Cloud Cover %</t>
+  </si>
+  <si>
+    <t>Precip %</t>
+  </si>
+  <si>
+    <t>Precip Inches</t>
+  </si>
+  <si>
+    <t>Visibility Miles</t>
+  </si>
+  <si>
+    <t>CAPE J/kg</t>
+  </si>
+  <si>
+    <t>Wind MPH</t>
+  </si>
+  <si>
+    <t>Wind Gust MPH</t>
+  </si>
+  <si>
+    <t>Wind From</t>
+  </si>
+  <si>
+    <t>Wind From Degrees</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Crosswind MPH</t>
+  </si>
+  <si>
+    <t>Effective Wind Vector MPH</t>
+  </si>
+  <si>
+    <t>Park Swirl Uncertainty MPH</t>
+  </si>
+  <si>
+    <t>LF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>CF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>RF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>Park Swirl Factor</t>
+  </si>
+  <si>
+    <t>Air Density kg/m3</t>
+  </si>
+  <si>
+    <t>Air Density Class</t>
+  </si>
+  <si>
+    <t>Density Altitude Ft</t>
+  </si>
+  <si>
+    <t>Roof Status</t>
+  </si>
+  <si>
+    <t>Roof Basis</t>
+  </si>
+  <si>
+    <t>HR Carry Score</t>
+  </si>
+  <si>
+    <t>Carry Multiplier</t>
+  </si>
+  <si>
+    <t>LHB Carry Score</t>
+  </si>
+  <si>
+    <t>RHB Carry Score</t>
+  </si>
+  <si>
+    <t>XBH Score</t>
+  </si>
+  <si>
+    <t>Run Environment Score</t>
+  </si>
+  <si>
+    <t>Pitching Comfort Score</t>
+  </si>
+  <si>
+    <t>Delay Risk Score</t>
+  </si>
+  <si>
+    <t>Delay Risk</t>
+  </si>
+  <si>
+    <t>NWS Temp F</t>
+  </si>
+  <si>
+    <t>Model Temp F</t>
+  </si>
+  <si>
+    <t>NWS Wind MPH</t>
+  </si>
+  <si>
+    <t>Model Wind MPH</t>
+  </si>
+  <si>
+    <t>First Pitch</t>
+  </si>
+  <si>
+    <t>+1 Hour</t>
+  </si>
+  <si>
+    <t>+2 Hours</t>
+  </si>
+  <si>
+    <t>+3 Hours</t>
   </si>
   <si>
     <t>07:10 PM EDT</t>
   </si>
   <si>
-    <t>Citizens Bank Park</t>
-  </si>
-  <si>
-    <t>OPEN</t>
-  </si>
-  <si>
-    <t>OPEN-AIR PARK</t>
-  </si>
-  <si>
-    <t>Mostly clear</t>
-  </si>
-  <si>
-    <t>🔴 5.1 mph In from LF</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>FORECAST MODEL</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>Density 86 | Wind 44 | Temp 71 | Altitude 66 | Confidence 90%</t>
-  </si>
-  <si>
-    <t>🟨 Neutral</t>
-  </si>
-  <si>
-    <t>IMPROVING</t>
-  </si>
-  <si>
-    <t>MODERATE</t>
-  </si>
-  <si>
-    <t>LOW</t>
-  </si>
-  <si>
-    <t>2026-07-16 12:30:07 AM PDT</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Target Local</t>
-  </si>
-  <si>
-    <t>Forecast Run UTC</t>
-  </si>
-  <si>
-    <t>NWS Forecast Updated</t>
-  </si>
-  <si>
-    <t>Hours Until Game</t>
-  </si>
-  <si>
-    <t>Temperature Model Spread F</t>
-  </si>
-  <si>
-    <t>Wind Model Spread MPH</t>
-  </si>
-  <si>
-    <t>Precip Model Spread Pct</t>
-  </si>
-  <si>
-    <t>Wind Direction Spread Degrees</t>
-  </si>
-  <si>
-    <t>Wind Toward CF Spread MPH</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing Out %</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing In %</t>
-  </si>
-  <si>
-    <t>Exact-Time Interpolation</t>
-  </si>
-  <si>
-    <t>Interpolation Lower Time</t>
-  </si>
-  <si>
-    <t>Interpolation Upper Time</t>
-  </si>
-  <si>
-    <t>Interpolation Fraction</t>
-  </si>
-  <si>
-    <t>Ensemble Disagreement Score</t>
-  </si>
-  <si>
-    <t>Weather Confidence %</t>
-  </si>
-  <si>
-    <t>Confidence-Adjusted HR Score</t>
-  </si>
-  <si>
-    <t>Park Wind Exposure</t>
-  </si>
-  <si>
-    <t>Park Temperature Offset F</t>
-  </si>
-  <si>
-    <t>Park Carry Bias</t>
-  </si>
-  <si>
-    <t>Microclimate Adjustment</t>
-  </si>
-  <si>
-    <t>Conditions</t>
-  </si>
-  <si>
-    <t>Temp F</t>
-  </si>
-  <si>
-    <t>Feels Like F</t>
-  </si>
-  <si>
-    <t>Dew Point F</t>
-  </si>
-  <si>
-    <t>RH %</t>
-  </si>
-  <si>
-    <t>Surface Pressure hPa</t>
-  </si>
-  <si>
-    <t>Sea Level Pressure hPa</t>
-  </si>
-  <si>
-    <t>Cloud Cover %</t>
-  </si>
-  <si>
-    <t>Precip %</t>
-  </si>
-  <si>
-    <t>Precip Inches</t>
-  </si>
-  <si>
-    <t>Visibility Miles</t>
-  </si>
-  <si>
-    <t>CAPE J/kg</t>
-  </si>
-  <si>
-    <t>Wind MPH</t>
-  </si>
-  <si>
-    <t>Wind Gust MPH</t>
-  </si>
-  <si>
-    <t>Wind From</t>
-  </si>
-  <si>
-    <t>Wind From Degrees</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Crosswind MPH</t>
-  </si>
-  <si>
-    <t>Effective Wind Vector MPH</t>
-  </si>
-  <si>
-    <t>Park Swirl Uncertainty MPH</t>
-  </si>
-  <si>
-    <t>LF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>CF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>RF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>Park Swirl Factor</t>
-  </si>
-  <si>
-    <t>Air Density kg/m3</t>
-  </si>
-  <si>
-    <t>Air Density Class</t>
-  </si>
-  <si>
-    <t>Density Altitude Ft</t>
-  </si>
-  <si>
-    <t>Roof Status</t>
-  </si>
-  <si>
-    <t>Roof Basis</t>
-  </si>
-  <si>
-    <t>HR Carry Score</t>
-  </si>
-  <si>
-    <t>Carry Multiplier</t>
-  </si>
-  <si>
-    <t>LHB Carry Score</t>
-  </si>
-  <si>
-    <t>RHB Carry Score</t>
-  </si>
-  <si>
-    <t>XBH Score</t>
-  </si>
-  <si>
-    <t>Run Environment Score</t>
-  </si>
-  <si>
-    <t>Pitching Comfort Score</t>
-  </si>
-  <si>
-    <t>Delay Risk Score</t>
-  </si>
-  <si>
-    <t>Delay Risk</t>
-  </si>
-  <si>
-    <t>NWS Temp F</t>
-  </si>
-  <si>
-    <t>Model Temp F</t>
-  </si>
-  <si>
-    <t>NWS Wind MPH</t>
-  </si>
-  <si>
-    <t>Model Wind MPH</t>
-  </si>
-  <si>
-    <t>First Pitch</t>
-  </si>
-  <si>
-    <t>+1 Hour</t>
-  </si>
-  <si>
-    <t>+2 Hours</t>
-  </si>
-  <si>
-    <t>+3 Hours</t>
-  </si>
-  <si>
     <t>08:10 PM EDT</t>
   </si>
   <si>
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>10:10 PM EDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 07:30:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-16T06:30:59+00:00</t>
+    <t>2026-07-16 20:24:56 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-16T08:08:16+00:00</t>
   </si>
   <si>
     <t>YES</t>
   </si>
   <si>
+    <t>2026-07-16T18:00</t>
+  </si>
+  <si>
     <t>2026-07-16T19:00</t>
   </si>
   <si>
@@ -489,9 +492,6 @@
   </si>
   <si>
     <t>2026-07-16T22:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T23:00</t>
   </si>
   <si>
     <t>WNW</t>
@@ -961,7 +961,7 @@
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="27.7109375" customWidth="1"/>
     <col min="12" max="12" width="33.7109375" customWidth="1"/>
-    <col min="13" max="13" width="22.7109375" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" customWidth="1"/>
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" customWidth="1"/>
@@ -985,7 +985,7 @@
     <col min="39" max="39" width="22.7109375" customWidth="1"/>
     <col min="40" max="40" width="17.7109375" customWidth="1"/>
     <col min="41" max="41" width="15.7109375" customWidth="1"/>
-    <col min="42" max="42" width="16.7109375" customWidth="1"/>
+    <col min="42" max="42" width="19.7109375" customWidth="1"/>
     <col min="43" max="43" width="34.7109375" customWidth="1"/>
     <col min="44" max="44" width="33.7109375" customWidth="1"/>
     <col min="45" max="45" width="32.7109375" customWidth="1"/>
@@ -1186,37 +1186,37 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>94.5</v>
+        <v>95.2</v>
       </c>
       <c r="L2">
-        <v>42</v>
+        <v>44.1</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>9.699999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>-5.1</v>
+        <v>-6</v>
       </c>
       <c r="Q2">
-        <v>-0.2</v>
+        <v>0.6</v>
       </c>
       <c r="R2">
-        <v>5.1</v>
+        <v>7.2</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
       </c>
       <c r="U2">
-        <v>23.2</v>
+        <v>26.4</v>
       </c>
       <c r="V2">
-        <v>59.1</v>
+        <v>60.8</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1225,61 +1225,61 @@
         <v>66</v>
       </c>
       <c r="Y2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Z2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AA2">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="AB2">
-        <v>89.5</v>
+        <v>88.5</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>-2.2</v>
+        <v>-0.8</v>
       </c>
       <c r="AE2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AF2">
-        <v>0</v>
+        <v>22.5</v>
       </c>
       <c r="AG2">
-        <v>90</v>
+        <v>60.7</v>
       </c>
       <c r="AH2">
-        <v>11.5</v>
+        <v>13.1</v>
       </c>
       <c r="AI2">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1385</v>
+        <v>1.1337</v>
       </c>
       <c r="AK2">
-        <v>2305</v>
+        <v>2419</v>
       </c>
       <c r="AL2">
-        <v>1008.8</v>
+        <v>1008.3</v>
       </c>
       <c r="AM2">
-        <v>64.8</v>
+        <v>68.2</v>
       </c>
       <c r="AN2">
-        <v>91.59999999999999</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="AO2">
-        <v>43.6</v>
+        <v>45.6</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>1.8</v>
+        <v>7.7</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1291,19 +1291,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>24</v>
+        <v>26.5</v>
       </c>
       <c r="AV2" t="s">
         <v>70</v>
       </c>
       <c r="AW2">
-        <v>10</v>
+        <v>17.4</v>
       </c>
       <c r="AX2" t="s">
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>59.1</v>
+        <v>736.7</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1371,7 +1371,7 @@
     <col min="28" max="28" width="27.7109375" customWidth="1"/>
     <col min="29" max="29" width="17.7109375" customWidth="1"/>
     <col min="30" max="30" width="25.7109375" customWidth="1"/>
-    <col min="31" max="31" width="14.7109375" customWidth="1"/>
+    <col min="31" max="31" width="12.7109375" customWidth="1"/>
     <col min="32" max="32" width="10.7109375" customWidth="1"/>
     <col min="33" max="33" width="14.7109375" customWidth="1"/>
     <col min="34" max="34" width="13.7109375" customWidth="1"/>
@@ -1680,34 +1680,34 @@
         <v>150</v>
       </c>
       <c r="J2">
-        <v>59.1</v>
+        <v>736.7</v>
       </c>
       <c r="K2">
-        <v>15.7</v>
+        <v>1.8</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>2.44</v>
+        <v>1.36</v>
       </c>
       <c r="N2">
-        <v>3.01</v>
+        <v>1.72</v>
       </c>
       <c r="O2">
-        <v>5.12</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="P2">
-        <v>9.5</v>
+        <v>11.2</v>
       </c>
       <c r="Q2">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>56.2</v>
       </c>
       <c r="S2">
-        <v>75</v>
+        <v>43.8</v>
       </c>
       <c r="T2" t="s">
         <v>151</v>
@@ -1722,13 +1722,13 @@
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>20.6</v>
+        <v>13.9</v>
       </c>
       <c r="Y2">
-        <v>88.40000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="Z2">
-        <v>67.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1746,76 +1746,76 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>94.5</v>
+        <v>95.2</v>
       </c>
       <c r="AG2">
-        <v>96.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="AH2">
-        <v>66.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AI2">
-        <v>42</v>
+        <v>44.1</v>
       </c>
       <c r="AJ2">
-        <v>1007.9</v>
+        <v>1007.6</v>
       </c>
       <c r="AK2">
-        <v>1010.2</v>
+        <v>1009.9</v>
       </c>
       <c r="AL2">
-        <v>36.6</v>
+        <v>17.2</v>
       </c>
       <c r="AM2">
-        <v>23.2</v>
+        <v>26.4</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>35.1</v>
+        <v>49.4</v>
       </c>
       <c r="AP2">
-        <v>1122</v>
+        <v>2114</v>
       </c>
       <c r="AQ2">
-        <v>9.699999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="AR2">
-        <v>20.6</v>
+        <v>21.2</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>281.1</v>
+        <v>277.1</v>
       </c>
       <c r="AU2">
-        <v>-0.2</v>
+        <v>0.7</v>
       </c>
       <c r="AV2">
-        <v>-5.7</v>
+        <v>-6.7</v>
       </c>
       <c r="AW2">
-        <v>5.4</v>
+        <v>7.8</v>
       </c>
       <c r="AX2">
-        <v>-0.2</v>
+        <v>0.6</v>
       </c>
       <c r="AY2">
-        <v>-5.1</v>
+        <v>-6</v>
       </c>
       <c r="AZ2">
-        <v>5.1</v>
+        <v>7.2</v>
       </c>
       <c r="BA2">
-        <v>9.5</v>
+        <v>12.3</v>
       </c>
       <c r="BB2">
-        <v>-0.1</v>
+        <v>0.6</v>
       </c>
       <c r="BC2">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="BD2">
         <v>0.9399999999999999</v>
@@ -1830,13 +1830,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.131</v>
+        <v>1.1282</v>
       </c>
       <c r="BI2" t="s">
         <v>159</v>
       </c>
       <c r="BJ2">
-        <v>2524</v>
+        <v>2582</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1845,49 +1845,49 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>70.2</v>
+        <v>76</v>
       </c>
       <c r="BN2">
-        <v>1.048</v>
+        <v>1.062</v>
       </c>
       <c r="BO2">
-        <v>74.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BP2">
-        <v>65.7</v>
+        <v>70</v>
       </c>
       <c r="BQ2">
-        <v>59.5</v>
+        <v>61.7</v>
       </c>
       <c r="BR2">
-        <v>56.3</v>
+        <v>57.2</v>
       </c>
       <c r="BS2">
-        <v>42.2</v>
+        <v>38.3</v>
       </c>
       <c r="BT2">
-        <v>24</v>
+        <v>26.5</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>4.3</v>
+        <v>17.4</v>
       </c>
       <c r="BW2" t="s">
         <v>70</v>
       </c>
       <c r="BX2">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="BY2">
-        <v>94.40000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="BZ2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="CA2">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1919,34 +1919,34 @@
         <v>150</v>
       </c>
       <c r="J3">
-        <v>59.1</v>
+        <v>736.7</v>
       </c>
       <c r="K3">
-        <v>16.7</v>
+        <v>2.8</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.61</v>
+        <v>1.7</v>
       </c>
       <c r="N3">
-        <v>2.86</v>
+        <v>1.92</v>
       </c>
       <c r="O3">
-        <v>4.98</v>
+        <v>7.37</v>
       </c>
       <c r="P3">
-        <v>13</v>
+        <v>14.9</v>
       </c>
       <c r="Q3">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R3">
         <v>0</v>
       </c>
       <c r="S3">
-        <v>100</v>
+        <v>43.8</v>
       </c>
       <c r="T3" t="s">
         <v>151</v>
@@ -1961,13 +1961,13 @@
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>16.8</v>
+        <v>15.2</v>
       </c>
       <c r="Y3">
-        <v>89.09999999999999</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="Z3">
-        <v>63.1</v>
+        <v>67.3</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1985,76 +1985,76 @@
         <v>61</v>
       </c>
       <c r="AF3">
-        <v>91.8</v>
+        <v>93.5</v>
       </c>
       <c r="AG3">
-        <v>91.2</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AH3">
-        <v>64.09999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="AI3">
-        <v>42.5</v>
+        <v>45.4</v>
       </c>
       <c r="AJ3">
-        <v>1008.7</v>
+        <v>1008.1</v>
       </c>
       <c r="AK3">
-        <v>1010.9</v>
+        <v>1010.4</v>
       </c>
       <c r="AL3">
-        <v>40</v>
+        <v>20.5</v>
       </c>
       <c r="AM3">
-        <v>20</v>
+        <v>23.2</v>
       </c>
       <c r="AN3">
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>38.4</v>
+        <v>33.6</v>
       </c>
       <c r="AP3">
-        <v>358</v>
+        <v>1567</v>
       </c>
       <c r="AQ3">
-        <v>8.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AR3">
-        <v>20.2</v>
+        <v>19.7</v>
       </c>
       <c r="AS3" t="s">
         <v>157</v>
       </c>
       <c r="AT3">
-        <v>291</v>
+        <v>284.1</v>
       </c>
       <c r="AU3">
-        <v>-1.6</v>
+        <v>-0.7</v>
       </c>
       <c r="AV3">
-        <v>-6.2</v>
+        <v>-6.1</v>
       </c>
       <c r="AW3">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="AX3">
-        <v>-1.6</v>
+        <v>-0.7</v>
       </c>
       <c r="AY3">
         <v>-5.5</v>
       </c>
       <c r="AZ3">
-        <v>3.3</v>
+        <v>4.7</v>
       </c>
       <c r="BA3">
-        <v>8.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="BB3">
-        <v>-1.4</v>
+        <v>-0.6</v>
       </c>
       <c r="BC3">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="BD3">
         <v>0.9399999999999999</v>
@@ -2069,13 +2069,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1382</v>
+        <v>1.1327</v>
       </c>
       <c r="BI3" t="s">
         <v>159</v>
       </c>
       <c r="BJ3">
-        <v>2317</v>
+        <v>2449</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2084,49 +2084,49 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>64.7</v>
+        <v>68.7</v>
       </c>
       <c r="BN3">
-        <v>1.035</v>
+        <v>1.045</v>
       </c>
       <c r="BO3">
-        <v>68.90000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="BP3">
-        <v>61</v>
+        <v>64.3</v>
       </c>
       <c r="BQ3">
-        <v>57.5</v>
+        <v>59</v>
       </c>
       <c r="BR3">
-        <v>54.7</v>
+        <v>56.1</v>
       </c>
       <c r="BS3">
-        <v>46.9</v>
+        <v>42.4</v>
       </c>
       <c r="BT3">
-        <v>14.6</v>
+        <v>24.8</v>
       </c>
       <c r="BU3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BV3">
-        <v>6</v>
+        <v>1.1</v>
       </c>
       <c r="BW3" t="s">
         <v>70</v>
       </c>
       <c r="BX3">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="BY3">
-        <v>91.09999999999999</v>
+        <v>92.7</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>7.8</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2158,28 +2158,28 @@
         <v>150</v>
       </c>
       <c r="J4">
-        <v>59.1</v>
+        <v>736.7</v>
       </c>
       <c r="K4">
-        <v>17.7</v>
+        <v>3.8</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>0.79</v>
+        <v>1.43</v>
       </c>
       <c r="N4">
-        <v>2.23</v>
+        <v>1.34</v>
       </c>
       <c r="O4">
-        <v>3.61</v>
+        <v>6.73</v>
       </c>
       <c r="P4">
-        <v>12.1</v>
+        <v>18.2</v>
       </c>
       <c r="Q4">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -2200,13 +2200,13 @@
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>11.1</v>
+        <v>12.1</v>
       </c>
       <c r="Y4">
-        <v>91</v>
+        <v>90.5</v>
       </c>
       <c r="Z4">
-        <v>51.1</v>
+        <v>63.2</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2224,73 +2224,73 @@
         <v>61</v>
       </c>
       <c r="AF4">
-        <v>88.59999999999999</v>
+        <v>91</v>
       </c>
       <c r="AG4">
-        <v>87.8</v>
+        <v>92.8</v>
       </c>
       <c r="AH4">
-        <v>63.8</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AI4">
-        <v>46.5</v>
+        <v>46.6</v>
       </c>
       <c r="AJ4">
-        <v>1009.6</v>
+        <v>1009</v>
       </c>
       <c r="AK4">
-        <v>1011.8</v>
+        <v>1011.3</v>
       </c>
       <c r="AL4">
-        <v>39.5</v>
+        <v>19.9</v>
       </c>
       <c r="AM4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AN4">
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>25.2</v>
+        <v>32.6</v>
       </c>
       <c r="AP4">
-        <v>154</v>
+        <v>1139</v>
       </c>
       <c r="AQ4">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
       <c r="AR4">
-        <v>18.8</v>
+        <v>17.7</v>
       </c>
       <c r="AS4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AT4">
-        <v>329.2</v>
+        <v>292</v>
       </c>
       <c r="AU4">
+        <v>-1.8</v>
+      </c>
+      <c r="AV4">
         <v>-6.3</v>
       </c>
-      <c r="AV4">
-        <v>-8.300000000000001</v>
-      </c>
       <c r="AW4">
-        <v>-2</v>
+        <v>3.4</v>
       </c>
       <c r="AX4">
-        <v>-6.2</v>
+        <v>-1.7</v>
       </c>
       <c r="AY4">
-        <v>-7.4</v>
+        <v>-5.6</v>
       </c>
       <c r="AZ4">
-        <v>-1.9</v>
+        <v>3.1</v>
       </c>
       <c r="BA4">
-        <v>5.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BB4">
-        <v>-5.5</v>
+        <v>-1.5</v>
       </c>
       <c r="BC4">
         <v>0.8</v>
@@ -2308,13 +2308,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.146</v>
+        <v>1.1394</v>
       </c>
       <c r="BI4" t="s">
         <v>159</v>
       </c>
       <c r="BJ4">
-        <v>2075</v>
+        <v>2253</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2323,49 +2323,49 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>51.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="BN4">
-        <v>1.003</v>
+        <v>1.035</v>
       </c>
       <c r="BO4">
-        <v>54.4</v>
+        <v>68.7</v>
       </c>
       <c r="BP4">
-        <v>49.4</v>
+        <v>60.9</v>
       </c>
       <c r="BQ4">
-        <v>52.5</v>
+        <v>57.2</v>
       </c>
       <c r="BR4">
-        <v>51.9</v>
+        <v>54.8</v>
       </c>
       <c r="BS4">
-        <v>51.6</v>
+        <v>48</v>
       </c>
       <c r="BT4">
-        <v>10.3</v>
+        <v>22.4</v>
       </c>
       <c r="BU4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BV4">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="BW4" t="s">
         <v>70</v>
       </c>
       <c r="BX4">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="BY4">
-        <v>87.8</v>
+        <v>89.8</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>7.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2397,28 +2397,28 @@
         <v>150</v>
       </c>
       <c r="J5">
-        <v>59.1</v>
+        <v>736.7</v>
       </c>
       <c r="K5">
-        <v>18.7</v>
+        <v>4.8</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.15</v>
+        <v>1.03</v>
       </c>
       <c r="N5">
-        <v>1.16</v>
+        <v>1.36</v>
       </c>
       <c r="O5">
-        <v>1.95</v>
+        <v>4.26</v>
       </c>
       <c r="P5">
-        <v>13.3</v>
+        <v>5.1</v>
       </c>
       <c r="Q5">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -2439,13 +2439,13 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>4.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="Y5">
-        <v>92.40000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="Z5">
-        <v>46.4</v>
+        <v>52.4</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2463,76 +2463,76 @@
         <v>61</v>
       </c>
       <c r="AF5">
-        <v>85.7</v>
+        <v>87.7</v>
       </c>
       <c r="AG5">
-        <v>82.8</v>
+        <v>88</v>
       </c>
       <c r="AH5">
-        <v>61.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AI5">
-        <v>47.5</v>
+        <v>49.9</v>
       </c>
       <c r="AJ5">
-        <v>1010.6</v>
+        <v>1009.9</v>
       </c>
       <c r="AK5">
-        <v>1012.8</v>
+        <v>1012.2</v>
       </c>
       <c r="AL5">
-        <v>40.5</v>
+        <v>27.1</v>
       </c>
       <c r="AM5">
-        <v>12.8</v>
+        <v>16</v>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>11.4</v>
+        <v>39.1</v>
       </c>
       <c r="AP5">
-        <v>35</v>
+        <v>517</v>
       </c>
       <c r="AQ5">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="AR5">
-        <v>18.5</v>
+        <v>14.1</v>
       </c>
       <c r="AS5" t="s">
         <v>158</v>
       </c>
       <c r="AT5">
-        <v>343.1</v>
+        <v>327.3</v>
       </c>
       <c r="AU5">
-        <v>-7.6</v>
+        <v>-5.8</v>
       </c>
       <c r="AV5">
-        <v>-8.4</v>
+        <v>-7.9</v>
       </c>
       <c r="AW5">
-        <v>-4</v>
+        <v>-1.7</v>
       </c>
       <c r="AX5">
-        <v>-7.4</v>
+        <v>-5.7</v>
       </c>
       <c r="AY5">
-        <v>-7.5</v>
+        <v>-7</v>
       </c>
       <c r="AZ5">
-        <v>-3.7</v>
+        <v>-1.6</v>
       </c>
       <c r="BA5">
-        <v>3.8</v>
+        <v>5.3</v>
       </c>
       <c r="BB5">
-        <v>-6.6</v>
+        <v>-5.1</v>
       </c>
       <c r="BC5">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="BD5">
         <v>0.9399999999999999</v>
@@ -2547,13 +2547,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.1539</v>
+        <v>1.1477</v>
       </c>
       <c r="BI5" t="s">
         <v>159</v>
       </c>
       <c r="BJ5">
-        <v>1850</v>
+        <v>2007</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2562,49 +2562,49 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>46.1</v>
+        <v>52.7</v>
       </c>
       <c r="BN5">
-        <v>0.991</v>
+        <v>1.007</v>
       </c>
       <c r="BO5">
-        <v>48.7</v>
+        <v>55.9</v>
       </c>
       <c r="BP5">
-        <v>45.3</v>
+        <v>50.9</v>
       </c>
       <c r="BQ5">
-        <v>50.4</v>
+        <v>52.6</v>
       </c>
       <c r="BR5">
-        <v>50.5</v>
+        <v>52.2</v>
       </c>
       <c r="BS5">
-        <v>55</v>
+        <v>55.1</v>
       </c>
       <c r="BT5">
-        <v>7.4</v>
+        <v>14</v>
       </c>
       <c r="BU5" t="s">
         <v>70</v>
       </c>
       <c r="BV5">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="BW5" t="s">
         <v>70</v>
       </c>
       <c r="BX5">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="BY5">
-        <v>84.2</v>
+        <v>86.3</v>
       </c>
       <c r="BZ5">
         <v>10</v>
       </c>
       <c r="CA5">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
     </row>
   </sheetData>
@@ -2706,34 +2706,34 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>59.1</v>
+        <v>60.8</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>89.5</v>
+        <v>88.5</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="K2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="L2" t="s">
         <v>67</v>
       </c>
       <c r="M2">
-        <v>91.59999999999999</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="N2">
-        <v>2305</v>
+        <v>2419</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 01:53 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="161">
   <si>
     <t>Date</t>
   </si>
@@ -209,7 +209,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 7.2 mph Out to RF</t>
+    <t>🟢 8.7 mph Out to RF</t>
   </si>
   <si>
     <t>W</t>
@@ -221,7 +221,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 88 | Wind 48 | Temp 72 | Altitude 67 | Confidence 88%</t>
+    <t>Density 87 | Wind 55 | Temp 70 | Altitude 66 | Confidence 81%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -233,274 +233,277 @@
     <t>MODERATE</t>
   </si>
   <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>2026-07-16 01:53:36 PM PDT</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Target Local</t>
+  </si>
+  <si>
+    <t>Forecast Run UTC</t>
+  </si>
+  <si>
+    <t>NWS Forecast Updated</t>
+  </si>
+  <si>
+    <t>Hours Until Game</t>
+  </si>
+  <si>
+    <t>Temperature Model Spread F</t>
+  </si>
+  <si>
+    <t>Wind Model Spread MPH</t>
+  </si>
+  <si>
+    <t>Precip Model Spread Pct</t>
+  </si>
+  <si>
+    <t>Wind Direction Spread Degrees</t>
+  </si>
+  <si>
+    <t>Wind Toward CF Spread MPH</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing Out %</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing In %</t>
+  </si>
+  <si>
+    <t>Exact-Time Interpolation</t>
+  </si>
+  <si>
+    <t>Interpolation Lower Time</t>
+  </si>
+  <si>
+    <t>Interpolation Upper Time</t>
+  </si>
+  <si>
+    <t>Interpolation Fraction</t>
+  </si>
+  <si>
+    <t>Ensemble Disagreement Score</t>
+  </si>
+  <si>
+    <t>Weather Confidence %</t>
+  </si>
+  <si>
+    <t>Confidence-Adjusted HR Score</t>
+  </si>
+  <si>
+    <t>Park Wind Exposure</t>
+  </si>
+  <si>
+    <t>Park Temperature Offset F</t>
+  </si>
+  <si>
+    <t>Park Carry Bias</t>
+  </si>
+  <si>
+    <t>Microclimate Adjustment</t>
+  </si>
+  <si>
+    <t>Conditions</t>
+  </si>
+  <si>
+    <t>Temp F</t>
+  </si>
+  <si>
+    <t>Feels Like F</t>
+  </si>
+  <si>
+    <t>Dew Point F</t>
+  </si>
+  <si>
+    <t>RH %</t>
+  </si>
+  <si>
+    <t>Surface Pressure hPa</t>
+  </si>
+  <si>
+    <t>Sea Level Pressure hPa</t>
+  </si>
+  <si>
+    <t>Cloud Cover %</t>
+  </si>
+  <si>
+    <t>Precip %</t>
+  </si>
+  <si>
+    <t>Precip Inches</t>
+  </si>
+  <si>
+    <t>Visibility Miles</t>
+  </si>
+  <si>
+    <t>CAPE J/kg</t>
+  </si>
+  <si>
+    <t>Wind MPH</t>
+  </si>
+  <si>
+    <t>Wind Gust MPH</t>
+  </si>
+  <si>
+    <t>Wind From</t>
+  </si>
+  <si>
+    <t>Wind From Degrees</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Crosswind MPH</t>
+  </si>
+  <si>
+    <t>Effective Wind Vector MPH</t>
+  </si>
+  <si>
+    <t>Park Swirl Uncertainty MPH</t>
+  </si>
+  <si>
+    <t>LF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>CF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>RF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>Park Swirl Factor</t>
+  </si>
+  <si>
+    <t>Air Density kg/m3</t>
+  </si>
+  <si>
+    <t>Air Density Class</t>
+  </si>
+  <si>
+    <t>Density Altitude Ft</t>
+  </si>
+  <si>
+    <t>Roof Status</t>
+  </si>
+  <si>
+    <t>Roof Basis</t>
+  </si>
+  <si>
+    <t>HR Carry Score</t>
+  </si>
+  <si>
+    <t>Carry Multiplier</t>
+  </si>
+  <si>
+    <t>LHB Carry Score</t>
+  </si>
+  <si>
+    <t>RHB Carry Score</t>
+  </si>
+  <si>
+    <t>XBH Score</t>
+  </si>
+  <si>
+    <t>Run Environment Score</t>
+  </si>
+  <si>
+    <t>Pitching Comfort Score</t>
+  </si>
+  <si>
+    <t>Delay Risk Score</t>
+  </si>
+  <si>
+    <t>Delay Risk</t>
+  </si>
+  <si>
+    <t>NWS Temp F</t>
+  </si>
+  <si>
+    <t>Model Temp F</t>
+  </si>
+  <si>
+    <t>NWS Wind MPH</t>
+  </si>
+  <si>
+    <t>Model Wind MPH</t>
+  </si>
+  <si>
+    <t>First Pitch</t>
+  </si>
+  <si>
+    <t>+1 Hour</t>
+  </si>
+  <si>
+    <t>+2 Hours</t>
+  </si>
+  <si>
+    <t>+3 Hours</t>
+  </si>
+  <si>
+    <t>07:10 PM EDT</t>
+  </si>
+  <si>
+    <t>08:10 PM EDT</t>
+  </si>
+  <si>
+    <t>09:10 PM EDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 20:53:36 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-16T08:08:16+00:00</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>2026-07-16T18:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T19:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T20:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T21:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T22:00</t>
+  </si>
+  <si>
+    <t>Partly cloudy</t>
+  </si>
+  <si>
+    <t>WNW</t>
+  </si>
+  <si>
+    <t>LIGHT</t>
+  </si>
+  <si>
     <t>LOW</t>
-  </si>
-  <si>
-    <t>2026-07-16 01:24:56 PM PDT</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Target Local</t>
-  </si>
-  <si>
-    <t>Forecast Run UTC</t>
-  </si>
-  <si>
-    <t>NWS Forecast Updated</t>
-  </si>
-  <si>
-    <t>Hours Until Game</t>
-  </si>
-  <si>
-    <t>Temperature Model Spread F</t>
-  </si>
-  <si>
-    <t>Wind Model Spread MPH</t>
-  </si>
-  <si>
-    <t>Precip Model Spread Pct</t>
-  </si>
-  <si>
-    <t>Wind Direction Spread Degrees</t>
-  </si>
-  <si>
-    <t>Wind Toward CF Spread MPH</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing Out %</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing In %</t>
-  </si>
-  <si>
-    <t>Exact-Time Interpolation</t>
-  </si>
-  <si>
-    <t>Interpolation Lower Time</t>
-  </si>
-  <si>
-    <t>Interpolation Upper Time</t>
-  </si>
-  <si>
-    <t>Interpolation Fraction</t>
-  </si>
-  <si>
-    <t>Ensemble Disagreement Score</t>
-  </si>
-  <si>
-    <t>Weather Confidence %</t>
-  </si>
-  <si>
-    <t>Confidence-Adjusted HR Score</t>
-  </si>
-  <si>
-    <t>Park Wind Exposure</t>
-  </si>
-  <si>
-    <t>Park Temperature Offset F</t>
-  </si>
-  <si>
-    <t>Park Carry Bias</t>
-  </si>
-  <si>
-    <t>Microclimate Adjustment</t>
-  </si>
-  <si>
-    <t>Conditions</t>
-  </si>
-  <si>
-    <t>Temp F</t>
-  </si>
-  <si>
-    <t>Feels Like F</t>
-  </si>
-  <si>
-    <t>Dew Point F</t>
-  </si>
-  <si>
-    <t>RH %</t>
-  </si>
-  <si>
-    <t>Surface Pressure hPa</t>
-  </si>
-  <si>
-    <t>Sea Level Pressure hPa</t>
-  </si>
-  <si>
-    <t>Cloud Cover %</t>
-  </si>
-  <si>
-    <t>Precip %</t>
-  </si>
-  <si>
-    <t>Precip Inches</t>
-  </si>
-  <si>
-    <t>Visibility Miles</t>
-  </si>
-  <si>
-    <t>CAPE J/kg</t>
-  </si>
-  <si>
-    <t>Wind MPH</t>
-  </si>
-  <si>
-    <t>Wind Gust MPH</t>
-  </si>
-  <si>
-    <t>Wind From</t>
-  </si>
-  <si>
-    <t>Wind From Degrees</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Crosswind MPH</t>
-  </si>
-  <si>
-    <t>Effective Wind Vector MPH</t>
-  </si>
-  <si>
-    <t>Park Swirl Uncertainty MPH</t>
-  </si>
-  <si>
-    <t>LF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>CF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>RF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>Park Swirl Factor</t>
-  </si>
-  <si>
-    <t>Air Density kg/m3</t>
-  </si>
-  <si>
-    <t>Air Density Class</t>
-  </si>
-  <si>
-    <t>Density Altitude Ft</t>
-  </si>
-  <si>
-    <t>Roof Status</t>
-  </si>
-  <si>
-    <t>Roof Basis</t>
-  </si>
-  <si>
-    <t>HR Carry Score</t>
-  </si>
-  <si>
-    <t>Carry Multiplier</t>
-  </si>
-  <si>
-    <t>LHB Carry Score</t>
-  </si>
-  <si>
-    <t>RHB Carry Score</t>
-  </si>
-  <si>
-    <t>XBH Score</t>
-  </si>
-  <si>
-    <t>Run Environment Score</t>
-  </si>
-  <si>
-    <t>Pitching Comfort Score</t>
-  </si>
-  <si>
-    <t>Delay Risk Score</t>
-  </si>
-  <si>
-    <t>Delay Risk</t>
-  </si>
-  <si>
-    <t>NWS Temp F</t>
-  </si>
-  <si>
-    <t>Model Temp F</t>
-  </si>
-  <si>
-    <t>NWS Wind MPH</t>
-  </si>
-  <si>
-    <t>Model Wind MPH</t>
-  </si>
-  <si>
-    <t>First Pitch</t>
-  </si>
-  <si>
-    <t>+1 Hour</t>
-  </si>
-  <si>
-    <t>+2 Hours</t>
-  </si>
-  <si>
-    <t>+3 Hours</t>
-  </si>
-  <si>
-    <t>07:10 PM EDT</t>
-  </si>
-  <si>
-    <t>08:10 PM EDT</t>
-  </si>
-  <si>
-    <t>09:10 PM EDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 20:24:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-16T08:08:16+00:00</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>2026-07-16T18:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T19:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T20:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T21:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T22:00</t>
-  </si>
-  <si>
-    <t>WNW</t>
-  </si>
-  <si>
-    <t>NNW</t>
-  </si>
-  <si>
-    <t>LIGHT</t>
   </si>
 </sst>
 </file>
@@ -1186,28 +1189,28 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>95.2</v>
+        <v>92.8</v>
       </c>
       <c r="L2">
-        <v>44.1</v>
+        <v>50.3</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>12.6</v>
+        <v>11.7</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>-6</v>
+        <v>-3.1</v>
       </c>
       <c r="Q2">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="R2">
-        <v>7.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
@@ -1216,7 +1219,7 @@
         <v>26.4</v>
       </c>
       <c r="V2">
-        <v>60.8</v>
+        <v>61.9</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1231,55 +1234,55 @@
         <v>5</v>
       </c>
       <c r="AA2">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="AB2">
-        <v>88.5</v>
+        <v>80.8</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>-0.8</v>
+        <v>2.2</v>
       </c>
       <c r="AE2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF2">
-        <v>22.5</v>
+        <v>56.2</v>
       </c>
       <c r="AG2">
-        <v>60.7</v>
+        <v>43.8</v>
       </c>
       <c r="AH2">
-        <v>13.1</v>
+        <v>46.7</v>
       </c>
       <c r="AI2">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="AJ2">
-        <v>1.1337</v>
+        <v>1.1379</v>
       </c>
       <c r="AK2">
-        <v>2419</v>
+        <v>2253</v>
       </c>
       <c r="AL2">
-        <v>1008.3</v>
+        <v>1008.7</v>
       </c>
       <c r="AM2">
-        <v>68.2</v>
+        <v>71</v>
       </c>
       <c r="AN2">
-        <v>93.09999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="AO2">
-        <v>45.6</v>
+        <v>54.5</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>7.7</v>
+        <v>10</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1297,13 +1300,13 @@
         <v>70</v>
       </c>
       <c r="AW2">
-        <v>17.4</v>
+        <v>29.4</v>
       </c>
       <c r="AX2" t="s">
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>736.7</v>
+        <v>765.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1371,7 +1374,7 @@
     <col min="28" max="28" width="27.7109375" customWidth="1"/>
     <col min="29" max="29" width="17.7109375" customWidth="1"/>
     <col min="30" max="30" width="25.7109375" customWidth="1"/>
-    <col min="31" max="31" width="12.7109375" customWidth="1"/>
+    <col min="31" max="31" width="15.7109375" customWidth="1"/>
     <col min="32" max="32" width="10.7109375" customWidth="1"/>
     <col min="33" max="33" width="14.7109375" customWidth="1"/>
     <col min="34" max="34" width="13.7109375" customWidth="1"/>
@@ -1680,28 +1683,28 @@
         <v>150</v>
       </c>
       <c r="J2">
-        <v>736.7</v>
+        <v>765.3</v>
       </c>
       <c r="K2">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.36</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>1.72</v>
+        <v>0.18</v>
       </c>
       <c r="O2">
         <v>9.369999999999999</v>
       </c>
       <c r="P2">
-        <v>11.2</v>
+        <v>33.8</v>
       </c>
       <c r="Q2">
-        <v>1.7</v>
+        <v>4.2</v>
       </c>
       <c r="R2">
         <v>56.2</v>
@@ -1722,13 +1725,13 @@
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>13.9</v>
+        <v>15.8</v>
       </c>
       <c r="Y2">
-        <v>84.2</v>
+        <v>76.7</v>
       </c>
       <c r="Z2">
-        <v>71.90000000000001</v>
+        <v>73</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1746,25 +1749,25 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>95.2</v>
+        <v>92.8</v>
       </c>
       <c r="AG2">
-        <v>98.59999999999999</v>
+        <v>94.3</v>
       </c>
       <c r="AH2">
-        <v>69.40000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AI2">
-        <v>44.1</v>
+        <v>50.3</v>
       </c>
       <c r="AJ2">
-        <v>1007.6</v>
+        <v>1008</v>
       </c>
       <c r="AK2">
-        <v>1009.9</v>
+        <v>1010.3</v>
       </c>
       <c r="AL2">
-        <v>17.2</v>
+        <v>16.2</v>
       </c>
       <c r="AM2">
         <v>26.4</v>
@@ -1773,46 +1776,46 @@
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>49.4</v>
+        <v>50.3</v>
       </c>
       <c r="AP2">
-        <v>2114</v>
+        <v>2099</v>
       </c>
       <c r="AQ2">
-        <v>12.6</v>
+        <v>11.7</v>
       </c>
       <c r="AR2">
-        <v>21.2</v>
+        <v>18.9</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>277.1</v>
+        <v>262.4</v>
       </c>
       <c r="AU2">
-        <v>0.7</v>
+        <v>3.6</v>
       </c>
       <c r="AV2">
-        <v>-6.7</v>
+        <v>-3.5</v>
       </c>
       <c r="AW2">
-        <v>7.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AX2">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="AY2">
-        <v>-6</v>
+        <v>-3.1</v>
       </c>
       <c r="AZ2">
-        <v>7.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BA2">
-        <v>12.3</v>
+        <v>10.9</v>
       </c>
       <c r="BB2">
-        <v>0.6</v>
+        <v>3.2</v>
       </c>
       <c r="BC2">
         <v>1.1</v>
@@ -1830,13 +1833,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1282</v>
+        <v>1.1333</v>
       </c>
       <c r="BI2" t="s">
         <v>159</v>
       </c>
       <c r="BJ2">
-        <v>2582</v>
+        <v>2405</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1845,25 +1848,25 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>76</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="BN2">
-        <v>1.062</v>
+        <v>1.072</v>
       </c>
       <c r="BO2">
-        <v>81.90000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="BP2">
-        <v>70</v>
+        <v>74.3</v>
       </c>
       <c r="BQ2">
-        <v>61.7</v>
+        <v>62.1</v>
       </c>
       <c r="BR2">
-        <v>57.2</v>
+        <v>58</v>
       </c>
       <c r="BS2">
-        <v>38.3</v>
+        <v>41.8</v>
       </c>
       <c r="BT2">
         <v>26.5</v>
@@ -1872,7 +1875,7 @@
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>17.4</v>
+        <v>29.4</v>
       </c>
       <c r="BW2" t="s">
         <v>70</v>
@@ -1881,13 +1884,13 @@
         <v>95</v>
       </c>
       <c r="BY2">
-        <v>94.2</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="BZ2">
         <v>15</v>
       </c>
       <c r="CA2">
-        <v>11.2</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1919,31 +1922,31 @@
         <v>150</v>
       </c>
       <c r="J3">
-        <v>736.7</v>
+        <v>765.3</v>
       </c>
       <c r="K3">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.7</v>
+        <v>2.32</v>
       </c>
       <c r="N3">
-        <v>1.92</v>
+        <v>0.37</v>
       </c>
       <c r="O3">
         <v>7.37</v>
       </c>
       <c r="P3">
-        <v>14.9</v>
+        <v>48.9</v>
       </c>
       <c r="Q3">
-        <v>1.5</v>
+        <v>4.3</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>56.2</v>
       </c>
       <c r="S3">
         <v>43.8</v>
@@ -1961,13 +1964,13 @@
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>15.2</v>
+        <v>13</v>
       </c>
       <c r="Y3">
-        <v>92.59999999999999</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="Z3">
-        <v>67.3</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1985,25 +1988,25 @@
         <v>61</v>
       </c>
       <c r="AF3">
-        <v>93.5</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="AG3">
-        <v>96.40000000000001</v>
+        <v>96.7</v>
       </c>
       <c r="AH3">
-        <v>68.40000000000001</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="AI3">
-        <v>45.4</v>
+        <v>54.1</v>
       </c>
       <c r="AJ3">
-        <v>1008.1</v>
+        <v>1008.8</v>
       </c>
       <c r="AK3">
-        <v>1010.4</v>
+        <v>1011.1</v>
       </c>
       <c r="AL3">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="AM3">
         <v>23.2</v>
@@ -2012,49 +2015,49 @@
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>33.6</v>
+        <v>44.3</v>
       </c>
       <c r="AP3">
-        <v>1567</v>
+        <v>2771</v>
       </c>
       <c r="AQ3">
-        <v>9.800000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="AR3">
-        <v>19.7</v>
+        <v>15.4</v>
       </c>
       <c r="AS3" t="s">
-        <v>157</v>
+        <v>63</v>
       </c>
       <c r="AT3">
-        <v>284.1</v>
+        <v>262.1</v>
       </c>
       <c r="AU3">
-        <v>-0.7</v>
+        <v>2.6</v>
       </c>
       <c r="AV3">
-        <v>-6.1</v>
+        <v>-2.5</v>
       </c>
       <c r="AW3">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="AX3">
-        <v>-0.7</v>
+        <v>2.5</v>
       </c>
       <c r="AY3">
-        <v>-5.5</v>
+        <v>-2.2</v>
       </c>
       <c r="AZ3">
-        <v>4.7</v>
+        <v>6.3</v>
       </c>
       <c r="BA3">
-        <v>9.5</v>
+        <v>7.8</v>
       </c>
       <c r="BB3">
-        <v>-0.6</v>
+        <v>2.3</v>
       </c>
       <c r="BC3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="BD3">
         <v>0.9399999999999999</v>
@@ -2069,13 +2072,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1327</v>
+        <v>1.1365</v>
       </c>
       <c r="BI3" t="s">
         <v>159</v>
       </c>
       <c r="BJ3">
-        <v>2449</v>
+        <v>2290</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2084,25 +2087,25 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>68.7</v>
+        <v>76.3</v>
       </c>
       <c r="BN3">
-        <v>1.045</v>
+        <v>1.063</v>
       </c>
       <c r="BO3">
-        <v>73.40000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="BP3">
-        <v>64.3</v>
+        <v>72.2</v>
       </c>
       <c r="BQ3">
-        <v>59</v>
+        <v>59.6</v>
       </c>
       <c r="BR3">
-        <v>56.1</v>
+        <v>57.4</v>
       </c>
       <c r="BS3">
-        <v>42.4</v>
+        <v>45.2</v>
       </c>
       <c r="BT3">
         <v>24.8</v>
@@ -2111,22 +2114,22 @@
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>1.1</v>
+        <v>13.2</v>
       </c>
       <c r="BW3" t="s">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="BX3">
         <v>93</v>
       </c>
       <c r="BY3">
-        <v>92.7</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>9.9</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2158,34 +2161,34 @@
         <v>150</v>
       </c>
       <c r="J4">
-        <v>736.7</v>
+        <v>765.3</v>
       </c>
       <c r="K4">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.43</v>
+        <v>3.14</v>
       </c>
       <c r="N4">
-        <v>1.34</v>
+        <v>1.09</v>
       </c>
       <c r="O4">
         <v>6.73</v>
       </c>
       <c r="P4">
-        <v>18.2</v>
+        <v>57.5</v>
       </c>
       <c r="Q4">
-        <v>1.3</v>
+        <v>3.5</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>56.2</v>
       </c>
       <c r="S4">
-        <v>100</v>
+        <v>43.8</v>
       </c>
       <c r="T4" t="s">
         <v>151</v>
@@ -2200,13 +2203,13 @@
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>12.1</v>
+        <v>18.2</v>
       </c>
       <c r="Y4">
-        <v>90.5</v>
+        <v>80.2</v>
       </c>
       <c r="Z4">
-        <v>63.2</v>
+        <v>67.5</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2224,25 +2227,25 @@
         <v>61</v>
       </c>
       <c r="AF4">
-        <v>91</v>
+        <v>88.5</v>
       </c>
       <c r="AG4">
-        <v>92.8</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="AH4">
-        <v>66.90000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="AI4">
-        <v>46.6</v>
+        <v>58.7</v>
       </c>
       <c r="AJ4">
-        <v>1009</v>
+        <v>1009.3</v>
       </c>
       <c r="AK4">
-        <v>1011.3</v>
+        <v>1011.6</v>
       </c>
       <c r="AL4">
-        <v>19.9</v>
+        <v>30</v>
       </c>
       <c r="AM4">
         <v>20</v>
@@ -2251,49 +2254,49 @@
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>32.6</v>
+        <v>35.5</v>
       </c>
       <c r="AP4">
-        <v>1139</v>
+        <v>2277</v>
       </c>
       <c r="AQ4">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="AR4">
-        <v>17.7</v>
+        <v>12.5</v>
       </c>
       <c r="AS4" t="s">
-        <v>157</v>
+        <v>63</v>
       </c>
       <c r="AT4">
-        <v>292</v>
+        <v>266.7</v>
       </c>
       <c r="AU4">
-        <v>-1.8</v>
+        <v>1.7</v>
       </c>
       <c r="AV4">
-        <v>-6.3</v>
+        <v>-2.7</v>
       </c>
       <c r="AW4">
-        <v>3.4</v>
+        <v>5.4</v>
       </c>
       <c r="AX4">
-        <v>-1.7</v>
+        <v>1.6</v>
       </c>
       <c r="AY4">
-        <v>-5.6</v>
+        <v>-2.4</v>
       </c>
       <c r="AZ4">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="BA4">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="BB4">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="BC4">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BD4">
         <v>0.9399999999999999</v>
@@ -2308,13 +2311,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1394</v>
+        <v>1.1435</v>
       </c>
       <c r="BI4" t="s">
         <v>159</v>
       </c>
       <c r="BJ4">
-        <v>2253</v>
+        <v>2077</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2323,34 +2326,34 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>64.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="BN4">
-        <v>1.035</v>
+        <v>1.053</v>
       </c>
       <c r="BO4">
-        <v>68.7</v>
+        <v>75</v>
       </c>
       <c r="BP4">
-        <v>60.9</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="BQ4">
-        <v>57.2</v>
+        <v>57.9</v>
       </c>
       <c r="BR4">
-        <v>54.8</v>
+        <v>56.3</v>
       </c>
       <c r="BS4">
-        <v>48</v>
+        <v>49.2</v>
       </c>
       <c r="BT4">
-        <v>22.4</v>
+        <v>23</v>
       </c>
       <c r="BU4" t="s">
         <v>69</v>
       </c>
       <c r="BV4">
-        <v>7.4</v>
+        <v>21.2</v>
       </c>
       <c r="BW4" t="s">
         <v>70</v>
@@ -2359,13 +2362,13 @@
         <v>91</v>
       </c>
       <c r="BY4">
-        <v>89.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>7.7</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2397,34 +2400,34 @@
         <v>150</v>
       </c>
       <c r="J5">
-        <v>736.7</v>
+        <v>765.3</v>
       </c>
       <c r="K5">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.03</v>
+        <v>2.66</v>
       </c>
       <c r="N5">
-        <v>1.36</v>
+        <v>1.67</v>
       </c>
       <c r="O5">
         <v>4.26</v>
       </c>
       <c r="P5">
-        <v>5.1</v>
+        <v>70.3</v>
       </c>
       <c r="Q5">
-        <v>0.9</v>
+        <v>3.2</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>56.2</v>
       </c>
       <c r="S5">
-        <v>100</v>
+        <v>43.8</v>
       </c>
       <c r="T5" t="s">
         <v>151</v>
@@ -2439,13 +2442,13 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>9.699999999999999</v>
+        <v>17.2</v>
       </c>
       <c r="Y5">
-        <v>89.7</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="Z5">
-        <v>52.4</v>
+        <v>61.9</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2460,28 +2463,28 @@
         <v>1.6</v>
       </c>
       <c r="AE5" t="s">
-        <v>61</v>
+        <v>157</v>
       </c>
       <c r="AF5">
-        <v>87.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="AG5">
-        <v>88</v>
+        <v>91.8</v>
       </c>
       <c r="AH5">
-        <v>65.40000000000001</v>
+        <v>71</v>
       </c>
       <c r="AI5">
-        <v>49.9</v>
+        <v>63.6</v>
       </c>
       <c r="AJ5">
-        <v>1009.9</v>
+        <v>1010</v>
       </c>
       <c r="AK5">
-        <v>1012.2</v>
+        <v>1012.3</v>
       </c>
       <c r="AL5">
-        <v>27.1</v>
+        <v>61.6</v>
       </c>
       <c r="AM5">
         <v>16</v>
@@ -2490,49 +2493,49 @@
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>39.1</v>
+        <v>31.9</v>
       </c>
       <c r="AP5">
-        <v>517</v>
+        <v>2090</v>
       </c>
       <c r="AQ5">
-        <v>8</v>
+        <v>6.6</v>
       </c>
       <c r="AR5">
-        <v>14.1</v>
+        <v>12.2</v>
       </c>
       <c r="AS5" t="s">
         <v>158</v>
       </c>
       <c r="AT5">
-        <v>327.3</v>
+        <v>285.7</v>
       </c>
       <c r="AU5">
-        <v>-5.8</v>
+        <v>-0.6</v>
       </c>
       <c r="AV5">
-        <v>-7.9</v>
+        <v>-4.3</v>
       </c>
       <c r="AW5">
-        <v>-1.7</v>
+        <v>3.2</v>
       </c>
       <c r="AX5">
-        <v>-5.7</v>
+        <v>-0.6</v>
       </c>
       <c r="AY5">
-        <v>-7</v>
+        <v>-3.8</v>
       </c>
       <c r="AZ5">
-        <v>-1.6</v>
+        <v>3</v>
       </c>
       <c r="BA5">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="BB5">
-        <v>-5.1</v>
+        <v>-0.5</v>
       </c>
       <c r="BC5">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="BD5">
         <v>0.9399999999999999</v>
@@ -2547,13 +2550,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.1477</v>
+        <v>1.1497</v>
       </c>
       <c r="BI5" t="s">
         <v>159</v>
       </c>
       <c r="BJ5">
-        <v>2007</v>
+        <v>1883</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2562,34 +2565,34 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>52.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="BN5">
-        <v>1.007</v>
+        <v>1.036</v>
       </c>
       <c r="BO5">
-        <v>55.9</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="BP5">
-        <v>50.9</v>
+        <v>61.9</v>
       </c>
       <c r="BQ5">
-        <v>52.6</v>
+        <v>55.8</v>
       </c>
       <c r="BR5">
+        <v>54.7</v>
+      </c>
+      <c r="BS5">
         <v>52.2</v>
       </c>
-      <c r="BS5">
-        <v>55.1</v>
-      </c>
       <c r="BT5">
-        <v>14</v>
+        <v>20.8</v>
       </c>
       <c r="BU5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BV5">
-        <v>10.7</v>
+        <v>22.2</v>
       </c>
       <c r="BW5" t="s">
         <v>70</v>
@@ -2598,13 +2601,13 @@
         <v>88</v>
       </c>
       <c r="BY5">
-        <v>86.3</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="BZ5">
         <v>10</v>
       </c>
       <c r="CA5">
-        <v>6.6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2706,13 +2709,13 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>60.8</v>
+        <v>61.9</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>88.5</v>
+        <v>80.8</v>
       </c>
       <c r="H2">
         <v>7</v>
@@ -2721,19 +2724,19 @@
         <v>5</v>
       </c>
       <c r="J2">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="K2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L2" t="s">
         <v>67</v>
       </c>
       <c r="M2">
-        <v>93.09999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="N2">
-        <v>2419</v>
+        <v>2253</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 04:13 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -206,304 +206,304 @@
     <t>OPEN-AIR PARK</t>
   </si>
   <si>
+    <t>Partly cloudy</t>
+  </si>
+  <si>
+    <t>🟢 6.8 mph Out to RF</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>FORECAST MODEL</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>Density 87 | Wind 47 | Temp 70 | Altitude 66 | Confidence 88%</t>
+  </si>
+  <si>
+    <t>🟢 Good</t>
+  </si>
+  <si>
+    <t>IMPROVING</t>
+  </si>
+  <si>
+    <t>MODERATE</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>2026-07-16 04:13:23 PM PDT</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Target Local</t>
+  </si>
+  <si>
+    <t>Forecast Run UTC</t>
+  </si>
+  <si>
+    <t>NWS Forecast Updated</t>
+  </si>
+  <si>
+    <t>Hours Until Game</t>
+  </si>
+  <si>
+    <t>Temperature Model Spread F</t>
+  </si>
+  <si>
+    <t>Wind Model Spread MPH</t>
+  </si>
+  <si>
+    <t>Precip Model Spread Pct</t>
+  </si>
+  <si>
+    <t>Wind Direction Spread Degrees</t>
+  </si>
+  <si>
+    <t>Wind Toward CF Spread MPH</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing Out %</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing In %</t>
+  </si>
+  <si>
+    <t>Exact-Time Interpolation</t>
+  </si>
+  <si>
+    <t>Interpolation Lower Time</t>
+  </si>
+  <si>
+    <t>Interpolation Upper Time</t>
+  </si>
+  <si>
+    <t>Interpolation Fraction</t>
+  </si>
+  <si>
+    <t>Ensemble Disagreement Score</t>
+  </si>
+  <si>
+    <t>Weather Confidence %</t>
+  </si>
+  <si>
+    <t>Confidence-Adjusted HR Score</t>
+  </si>
+  <si>
+    <t>Park Wind Exposure</t>
+  </si>
+  <si>
+    <t>Park Temperature Offset F</t>
+  </si>
+  <si>
+    <t>Park Carry Bias</t>
+  </si>
+  <si>
+    <t>Microclimate Adjustment</t>
+  </si>
+  <si>
+    <t>Conditions</t>
+  </si>
+  <si>
+    <t>Temp F</t>
+  </si>
+  <si>
+    <t>Feels Like F</t>
+  </si>
+  <si>
+    <t>Dew Point F</t>
+  </si>
+  <si>
+    <t>RH %</t>
+  </si>
+  <si>
+    <t>Surface Pressure hPa</t>
+  </si>
+  <si>
+    <t>Sea Level Pressure hPa</t>
+  </si>
+  <si>
+    <t>Cloud Cover %</t>
+  </si>
+  <si>
+    <t>Precip %</t>
+  </si>
+  <si>
+    <t>Precip Inches</t>
+  </si>
+  <si>
+    <t>Visibility Miles</t>
+  </si>
+  <si>
+    <t>CAPE J/kg</t>
+  </si>
+  <si>
+    <t>Wind MPH</t>
+  </si>
+  <si>
+    <t>Wind Gust MPH</t>
+  </si>
+  <si>
+    <t>Wind From</t>
+  </si>
+  <si>
+    <t>Wind From Degrees</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Wind Toward RF MPH</t>
+  </si>
+  <si>
+    <t>Crosswind MPH</t>
+  </si>
+  <si>
+    <t>Effective Wind Vector MPH</t>
+  </si>
+  <si>
+    <t>Park Swirl Uncertainty MPH</t>
+  </si>
+  <si>
+    <t>LF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>CF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>RF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>Park Swirl Factor</t>
+  </si>
+  <si>
+    <t>Air Density kg/m3</t>
+  </si>
+  <si>
+    <t>Air Density Class</t>
+  </si>
+  <si>
+    <t>Density Altitude Ft</t>
+  </si>
+  <si>
+    <t>Roof Status</t>
+  </si>
+  <si>
+    <t>Roof Basis</t>
+  </si>
+  <si>
+    <t>HR Carry Score</t>
+  </si>
+  <si>
+    <t>Carry Multiplier</t>
+  </si>
+  <si>
+    <t>LHB Carry Score</t>
+  </si>
+  <si>
+    <t>RHB Carry Score</t>
+  </si>
+  <si>
+    <t>XBH Score</t>
+  </si>
+  <si>
+    <t>Run Environment Score</t>
+  </si>
+  <si>
+    <t>Pitching Comfort Score</t>
+  </si>
+  <si>
+    <t>Delay Risk Score</t>
+  </si>
+  <si>
+    <t>Delay Risk</t>
+  </si>
+  <si>
+    <t>NWS Temp F</t>
+  </si>
+  <si>
+    <t>Model Temp F</t>
+  </si>
+  <si>
+    <t>NWS Wind MPH</t>
+  </si>
+  <si>
+    <t>Model Wind MPH</t>
+  </si>
+  <si>
+    <t>First Pitch</t>
+  </si>
+  <si>
+    <t>+1 Hour</t>
+  </si>
+  <si>
+    <t>+2 Hours</t>
+  </si>
+  <si>
+    <t>+3 Hours</t>
+  </si>
+  <si>
+    <t>07:10 PM EDT</t>
+  </si>
+  <si>
+    <t>08:10 PM EDT</t>
+  </si>
+  <si>
+    <t>09:10 PM EDT</t>
+  </si>
+  <si>
+    <t>2026-07-16 23:13:23 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-16T20:08:51+00:00</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>2026-07-16T18:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T19:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T20:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T21:00</t>
+  </si>
+  <si>
+    <t>2026-07-16T22:00</t>
+  </si>
+  <si>
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.7 mph Out to RF</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>FORECAST MODEL</t>
-  </si>
-  <si>
-    <t>B+</t>
-  </si>
-  <si>
-    <t>Density 87 | Wind 55 | Temp 70 | Altitude 66 | Confidence 81%</t>
-  </si>
-  <si>
-    <t>🟢 Good</t>
-  </si>
-  <si>
-    <t>IMPROVING RAPIDLY</t>
-  </si>
-  <si>
-    <t>MODERATE</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>2026-07-16 01:53:36 PM PDT</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Target Local</t>
-  </si>
-  <si>
-    <t>Forecast Run UTC</t>
-  </si>
-  <si>
-    <t>NWS Forecast Updated</t>
-  </si>
-  <si>
-    <t>Hours Until Game</t>
-  </si>
-  <si>
-    <t>Temperature Model Spread F</t>
-  </si>
-  <si>
-    <t>Wind Model Spread MPH</t>
-  </si>
-  <si>
-    <t>Precip Model Spread Pct</t>
-  </si>
-  <si>
-    <t>Wind Direction Spread Degrees</t>
-  </si>
-  <si>
-    <t>Wind Toward CF Spread MPH</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing Out %</t>
-  </si>
-  <si>
-    <t>Probability Wind Blowing In %</t>
-  </si>
-  <si>
-    <t>Exact-Time Interpolation</t>
-  </si>
-  <si>
-    <t>Interpolation Lower Time</t>
-  </si>
-  <si>
-    <t>Interpolation Upper Time</t>
-  </si>
-  <si>
-    <t>Interpolation Fraction</t>
-  </si>
-  <si>
-    <t>Ensemble Disagreement Score</t>
-  </si>
-  <si>
-    <t>Weather Confidence %</t>
-  </si>
-  <si>
-    <t>Confidence-Adjusted HR Score</t>
-  </si>
-  <si>
-    <t>Park Wind Exposure</t>
-  </si>
-  <si>
-    <t>Park Temperature Offset F</t>
-  </si>
-  <si>
-    <t>Park Carry Bias</t>
-  </si>
-  <si>
-    <t>Microclimate Adjustment</t>
-  </si>
-  <si>
-    <t>Conditions</t>
-  </si>
-  <si>
-    <t>Temp F</t>
-  </si>
-  <si>
-    <t>Feels Like F</t>
-  </si>
-  <si>
-    <t>Dew Point F</t>
-  </si>
-  <si>
-    <t>RH %</t>
-  </si>
-  <si>
-    <t>Surface Pressure hPa</t>
-  </si>
-  <si>
-    <t>Sea Level Pressure hPa</t>
-  </si>
-  <si>
-    <t>Cloud Cover %</t>
-  </si>
-  <si>
-    <t>Precip %</t>
-  </si>
-  <si>
-    <t>Precip Inches</t>
-  </si>
-  <si>
-    <t>Visibility Miles</t>
-  </si>
-  <si>
-    <t>CAPE J/kg</t>
-  </si>
-  <si>
-    <t>Wind MPH</t>
-  </si>
-  <si>
-    <t>Wind Gust MPH</t>
-  </si>
-  <si>
-    <t>Wind From</t>
-  </si>
-  <si>
-    <t>Wind From Degrees</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Raw Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward CF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward LF MPH</t>
-  </si>
-  <si>
-    <t>Wind Toward RF MPH</t>
-  </si>
-  <si>
-    <t>Crosswind MPH</t>
-  </si>
-  <si>
-    <t>Effective Wind Vector MPH</t>
-  </si>
-  <si>
-    <t>Park Swirl Uncertainty MPH</t>
-  </si>
-  <si>
-    <t>LF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>CF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>RF Shield Multiplier</t>
-  </si>
-  <si>
-    <t>Park Swirl Factor</t>
-  </si>
-  <si>
-    <t>Air Density kg/m3</t>
-  </si>
-  <si>
-    <t>Air Density Class</t>
-  </si>
-  <si>
-    <t>Density Altitude Ft</t>
-  </si>
-  <si>
-    <t>Roof Status</t>
-  </si>
-  <si>
-    <t>Roof Basis</t>
-  </si>
-  <si>
-    <t>HR Carry Score</t>
-  </si>
-  <si>
-    <t>Carry Multiplier</t>
-  </si>
-  <si>
-    <t>LHB Carry Score</t>
-  </si>
-  <si>
-    <t>RHB Carry Score</t>
-  </si>
-  <si>
-    <t>XBH Score</t>
-  </si>
-  <si>
-    <t>Run Environment Score</t>
-  </si>
-  <si>
-    <t>Pitching Comfort Score</t>
-  </si>
-  <si>
-    <t>Delay Risk Score</t>
-  </si>
-  <si>
-    <t>Delay Risk</t>
-  </si>
-  <si>
-    <t>NWS Temp F</t>
-  </si>
-  <si>
-    <t>Model Temp F</t>
-  </si>
-  <si>
-    <t>NWS Wind MPH</t>
-  </si>
-  <si>
-    <t>Model Wind MPH</t>
-  </si>
-  <si>
-    <t>First Pitch</t>
-  </si>
-  <si>
-    <t>+1 Hour</t>
-  </si>
-  <si>
-    <t>+2 Hours</t>
-  </si>
-  <si>
-    <t>+3 Hours</t>
-  </si>
-  <si>
-    <t>07:10 PM EDT</t>
-  </si>
-  <si>
-    <t>08:10 PM EDT</t>
-  </si>
-  <si>
-    <t>09:10 PM EDT</t>
-  </si>
-  <si>
-    <t>2026-07-16 20:53:36 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-16T08:08:16+00:00</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>2026-07-16T18:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T19:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T20:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T21:00</t>
-  </si>
-  <si>
-    <t>2026-07-16T22:00</t>
-  </si>
-  <si>
-    <t>Partly cloudy</t>
-  </si>
-  <si>
     <t>WNW</t>
   </si>
   <si>
+    <t>N</t>
+  </si>
+  <si>
     <t>LIGHT</t>
-  </si>
-  <si>
-    <t>LOW</t>
   </si>
 </sst>
 </file>
@@ -988,7 +988,7 @@
     <col min="39" max="39" width="22.7109375" customWidth="1"/>
     <col min="40" max="40" width="17.7109375" customWidth="1"/>
     <col min="41" max="41" width="15.7109375" customWidth="1"/>
-    <col min="42" max="42" width="19.7109375" customWidth="1"/>
+    <col min="42" max="42" width="16.7109375" customWidth="1"/>
     <col min="43" max="43" width="34.7109375" customWidth="1"/>
     <col min="44" max="44" width="33.7109375" customWidth="1"/>
     <col min="45" max="45" width="32.7109375" customWidth="1"/>
@@ -1189,37 +1189,37 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>92.8</v>
+        <v>93.8</v>
       </c>
       <c r="L2">
-        <v>50.3</v>
+        <v>48.5</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>11.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>-3.1</v>
+        <v>-2.6</v>
       </c>
       <c r="Q2">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="R2">
-        <v>8.699999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
       </c>
       <c r="U2">
-        <v>26.4</v>
+        <v>22.4</v>
       </c>
       <c r="V2">
-        <v>61.9</v>
+        <v>60.1</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1228,61 +1228,61 @@
         <v>66</v>
       </c>
       <c r="Y2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Z2">
         <v>5</v>
       </c>
       <c r="AA2">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="AB2">
-        <v>80.8</v>
+        <v>88.2</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
+        <v>-1.2</v>
+      </c>
+      <c r="AE2">
+        <v>-1</v>
+      </c>
+      <c r="AF2">
+        <v>22.5</v>
+      </c>
+      <c r="AG2">
+        <v>77.5</v>
+      </c>
+      <c r="AH2">
+        <v>29.5</v>
+      </c>
+      <c r="AI2">
         <v>2.2</v>
       </c>
-      <c r="AE2">
-        <v>1</v>
-      </c>
-      <c r="AF2">
-        <v>56.2</v>
-      </c>
-      <c r="AG2">
-        <v>43.8</v>
-      </c>
-      <c r="AH2">
-        <v>46.7</v>
-      </c>
-      <c r="AI2">
-        <v>4</v>
-      </c>
       <c r="AJ2">
-        <v>1.1379</v>
+        <v>1.1367</v>
       </c>
       <c r="AK2">
-        <v>2253</v>
+        <v>2294</v>
       </c>
       <c r="AL2">
-        <v>1008.7</v>
+        <v>1008.5</v>
       </c>
       <c r="AM2">
-        <v>71</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AN2">
-        <v>90.8</v>
+        <v>91.3</v>
       </c>
       <c r="AO2">
-        <v>54.5</v>
+        <v>52.8</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1294,19 +1294,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>26.5</v>
+        <v>24.3</v>
       </c>
       <c r="AV2" t="s">
         <v>70</v>
       </c>
       <c r="AW2">
-        <v>29.4</v>
+        <v>17.9</v>
       </c>
       <c r="AX2" t="s">
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>765.3</v>
+        <v>184.5</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1683,28 +1683,28 @@
         <v>150</v>
       </c>
       <c r="J2">
-        <v>765.3</v>
+        <v>184.5</v>
       </c>
       <c r="K2">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>1.11</v>
       </c>
       <c r="N2">
-        <v>0.18</v>
+        <v>0.09</v>
       </c>
       <c r="O2">
-        <v>9.369999999999999</v>
+        <v>9.33</v>
       </c>
       <c r="P2">
-        <v>33.8</v>
+        <v>32.6</v>
       </c>
       <c r="Q2">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="R2">
         <v>56.2</v>
@@ -1725,13 +1725,13 @@
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>15.8</v>
+        <v>8</v>
       </c>
       <c r="Y2">
-        <v>76.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="Z2">
-        <v>73</v>
+        <v>76.2</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1749,76 +1749,76 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>92.8</v>
+        <v>93.8</v>
       </c>
       <c r="AG2">
-        <v>94.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="AH2">
-        <v>70.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AI2">
-        <v>50.3</v>
+        <v>48.5</v>
       </c>
       <c r="AJ2">
         <v>1008</v>
       </c>
       <c r="AK2">
-        <v>1010.3</v>
+        <v>1010.2</v>
       </c>
       <c r="AL2">
-        <v>16.2</v>
+        <v>72.5</v>
       </c>
       <c r="AM2">
-        <v>26.4</v>
+        <v>22.4</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>50.3</v>
+        <v>60.2</v>
       </c>
       <c r="AP2">
-        <v>2099</v>
+        <v>2705</v>
       </c>
       <c r="AQ2">
-        <v>11.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AR2">
-        <v>18.9</v>
+        <v>17.7</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>262.4</v>
+        <v>263.1</v>
       </c>
       <c r="AU2">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="AV2">
-        <v>-3.5</v>
+        <v>-2.9</v>
       </c>
       <c r="AW2">
-        <v>9.300000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="AX2">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="AY2">
-        <v>-3.1</v>
+        <v>-2.6</v>
       </c>
       <c r="AZ2">
-        <v>8.699999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="BA2">
-        <v>10.9</v>
+        <v>8.6</v>
       </c>
       <c r="BB2">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="BC2">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="BD2">
         <v>0.9399999999999999</v>
@@ -1833,13 +1833,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1333</v>
+        <v>1.1309</v>
       </c>
       <c r="BI2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BJ2">
-        <v>2405</v>
+        <v>2476</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1848,49 +1848,49 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>79.90000000000001</v>
+        <v>78</v>
       </c>
       <c r="BN2">
-        <v>1.072</v>
+        <v>1.067</v>
       </c>
       <c r="BO2">
-        <v>84.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BP2">
-        <v>74.3</v>
+        <v>73.5</v>
       </c>
       <c r="BQ2">
-        <v>62.1</v>
+        <v>60.6</v>
       </c>
       <c r="BR2">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="BS2">
-        <v>41.8</v>
+        <v>41.3</v>
       </c>
       <c r="BT2">
-        <v>26.5</v>
+        <v>24.3</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>29.4</v>
+        <v>5.1</v>
       </c>
       <c r="BW2" t="s">
         <v>70</v>
       </c>
       <c r="BX2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="BY2">
-        <v>89.90000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="BZ2">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="CA2">
-        <v>9.4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1922,34 +1922,34 @@
         <v>150</v>
       </c>
       <c r="J3">
-        <v>765.3</v>
+        <v>184.5</v>
       </c>
       <c r="K3">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>2.32</v>
+        <v>1.77</v>
       </c>
       <c r="N3">
-        <v>0.37</v>
+        <v>2.84</v>
       </c>
       <c r="O3">
-        <v>7.37</v>
+        <v>7.53</v>
       </c>
       <c r="P3">
-        <v>48.9</v>
+        <v>12</v>
       </c>
       <c r="Q3">
-        <v>4.3</v>
+        <v>0.9</v>
       </c>
       <c r="R3">
-        <v>56.2</v>
+        <v>0</v>
       </c>
       <c r="S3">
-        <v>43.8</v>
+        <v>100</v>
       </c>
       <c r="T3" t="s">
         <v>151</v>
@@ -1964,13 +1964,13 @@
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>13</v>
+        <v>18.2</v>
       </c>
       <c r="Y3">
-        <v>86.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="Z3">
-        <v>72.90000000000001</v>
+        <v>61</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1988,76 +1988,76 @@
         <v>61</v>
       </c>
       <c r="AF3">
-        <v>91.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="AG3">
-        <v>96.7</v>
+        <v>98.3</v>
       </c>
       <c r="AH3">
-        <v>71.59999999999999</v>
+        <v>70.5</v>
       </c>
       <c r="AI3">
-        <v>54.1</v>
+        <v>51.9</v>
       </c>
       <c r="AJ3">
-        <v>1008.8</v>
+        <v>1008.3</v>
       </c>
       <c r="AK3">
-        <v>1011.1</v>
+        <v>1010.6</v>
       </c>
       <c r="AL3">
-        <v>20.6</v>
+        <v>61.9</v>
       </c>
       <c r="AM3">
-        <v>23.2</v>
+        <v>17.4</v>
       </c>
       <c r="AN3">
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>44.3</v>
+        <v>53.7</v>
       </c>
       <c r="AP3">
-        <v>2771</v>
+        <v>2300</v>
       </c>
       <c r="AQ3">
-        <v>8.4</v>
+        <v>7</v>
       </c>
       <c r="AR3">
-        <v>15.4</v>
+        <v>13.1</v>
       </c>
       <c r="AS3" t="s">
-        <v>63</v>
+        <v>158</v>
       </c>
       <c r="AT3">
-        <v>262.1</v>
+        <v>302.1</v>
       </c>
       <c r="AU3">
-        <v>2.6</v>
+        <v>-2.6</v>
       </c>
       <c r="AV3">
-        <v>-2.5</v>
+        <v>-5.9</v>
       </c>
       <c r="AW3">
-        <v>6.7</v>
+        <v>1.6</v>
       </c>
       <c r="AX3">
-        <v>2.5</v>
+        <v>-2.6</v>
       </c>
       <c r="AY3">
-        <v>-2.2</v>
+        <v>-5.2</v>
       </c>
       <c r="AZ3">
+        <v>1.5</v>
+      </c>
+      <c r="BA3">
         <v>6.3</v>
       </c>
-      <c r="BA3">
-        <v>7.8</v>
-      </c>
       <c r="BB3">
-        <v>2.3</v>
+        <v>-2.3</v>
       </c>
       <c r="BC3">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BD3">
         <v>0.9399999999999999</v>
@@ -2072,13 +2072,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1365</v>
+        <v>1.1366</v>
       </c>
       <c r="BI3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BJ3">
-        <v>2290</v>
+        <v>2301</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2087,49 +2087,49 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>76.3</v>
+        <v>63.2</v>
       </c>
       <c r="BN3">
-        <v>1.063</v>
+        <v>1.032</v>
       </c>
       <c r="BO3">
-        <v>79.90000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="BP3">
-        <v>72.2</v>
+        <v>60.5</v>
       </c>
       <c r="BQ3">
-        <v>59.6</v>
+        <v>55.8</v>
       </c>
       <c r="BR3">
-        <v>57.4</v>
+        <v>55</v>
       </c>
       <c r="BS3">
-        <v>45.2</v>
+        <v>46.6</v>
       </c>
       <c r="BT3">
-        <v>24.8</v>
+        <v>21.6</v>
       </c>
       <c r="BU3" t="s">
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>13.2</v>
+        <v>15.2</v>
       </c>
       <c r="BW3" t="s">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="BX3">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="BY3">
-        <v>89.09999999999999</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>7.4</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2161,34 +2161,34 @@
         <v>150</v>
       </c>
       <c r="J4">
-        <v>765.3</v>
+        <v>184.5</v>
       </c>
       <c r="K4">
-        <v>3.3</v>
+        <v>0.9</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>3.14</v>
+        <v>1.61</v>
       </c>
       <c r="N4">
-        <v>1.09</v>
+        <v>2.15</v>
       </c>
       <c r="O4">
-        <v>6.73</v>
+        <v>6.66</v>
       </c>
       <c r="P4">
-        <v>57.5</v>
+        <v>46</v>
       </c>
       <c r="Q4">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="R4">
-        <v>56.2</v>
+        <v>0</v>
       </c>
       <c r="S4">
-        <v>43.8</v>
+        <v>100</v>
       </c>
       <c r="T4" t="s">
         <v>151</v>
@@ -2203,13 +2203,13 @@
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>18.2</v>
+        <v>15.2</v>
       </c>
       <c r="Y4">
-        <v>80.2</v>
+        <v>83.3</v>
       </c>
       <c r="Z4">
-        <v>67.5</v>
+        <v>52.7</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2224,76 +2224,76 @@
         <v>1.6</v>
       </c>
       <c r="AE4" t="s">
-        <v>61</v>
+        <v>157</v>
       </c>
       <c r="AF4">
-        <v>88.5</v>
+        <v>89</v>
       </c>
       <c r="AG4">
-        <v>92.90000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="AH4">
-        <v>71.09999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="AI4">
-        <v>58.7</v>
+        <v>57.4</v>
       </c>
       <c r="AJ4">
-        <v>1009.3</v>
+        <v>1009.2</v>
       </c>
       <c r="AK4">
-        <v>1011.6</v>
+        <v>1011.5</v>
       </c>
       <c r="AL4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AM4">
-        <v>20</v>
+        <v>10.6</v>
       </c>
       <c r="AN4">
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>35.5</v>
+        <v>43.7</v>
       </c>
       <c r="AP4">
-        <v>2277</v>
+        <v>2571</v>
       </c>
       <c r="AQ4">
-        <v>7.2</v>
+        <v>6.6</v>
       </c>
       <c r="AR4">
-        <v>12.5</v>
+        <v>9.4</v>
       </c>
       <c r="AS4" t="s">
-        <v>63</v>
+        <v>159</v>
       </c>
       <c r="AT4">
-        <v>266.7</v>
+        <v>352</v>
       </c>
       <c r="AU4">
-        <v>1.7</v>
+        <v>-6.2</v>
       </c>
       <c r="AV4">
-        <v>-2.7</v>
+        <v>-6.3</v>
       </c>
       <c r="AW4">
-        <v>5.4</v>
+        <v>-3.9</v>
       </c>
       <c r="AX4">
-        <v>1.6</v>
+        <v>-6.1</v>
       </c>
       <c r="AY4">
-        <v>-2.4</v>
+        <v>-5.6</v>
       </c>
       <c r="AZ4">
-        <v>5</v>
+        <v>-3.7</v>
       </c>
       <c r="BA4">
-        <v>6.8</v>
+        <v>2</v>
       </c>
       <c r="BB4">
-        <v>1.5</v>
+        <v>-5.5</v>
       </c>
       <c r="BC4">
         <v>0.6</v>
@@ -2311,13 +2311,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1435</v>
+        <v>1.1421</v>
       </c>
       <c r="BI4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BJ4">
-        <v>2077</v>
+        <v>2117</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2326,49 +2326,49 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>71.90000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="BN4">
-        <v>1.053</v>
+        <v>1.008</v>
       </c>
       <c r="BO4">
-        <v>75</v>
+        <v>54.9</v>
       </c>
       <c r="BP4">
-        <v>68.40000000000001</v>
+        <v>53.1</v>
       </c>
       <c r="BQ4">
-        <v>57.9</v>
+        <v>50.9</v>
       </c>
       <c r="BR4">
-        <v>56.3</v>
+        <v>53</v>
       </c>
       <c r="BS4">
-        <v>49.2</v>
+        <v>48.5</v>
       </c>
       <c r="BT4">
-        <v>23</v>
+        <v>17.8</v>
       </c>
       <c r="BU4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BV4">
-        <v>21.2</v>
+        <v>17.9</v>
       </c>
       <c r="BW4" t="s">
         <v>70</v>
       </c>
       <c r="BX4">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="BY4">
-        <v>85.40000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>5.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2400,34 +2400,34 @@
         <v>150</v>
       </c>
       <c r="J5">
-        <v>765.3</v>
+        <v>184.5</v>
       </c>
       <c r="K5">
-        <v>4.3</v>
+        <v>1.9</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>2.66</v>
+        <v>1.67</v>
       </c>
       <c r="N5">
-        <v>1.67</v>
+        <v>1.43</v>
       </c>
       <c r="O5">
         <v>4.26</v>
       </c>
       <c r="P5">
-        <v>70.3</v>
+        <v>37</v>
       </c>
       <c r="Q5">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="R5">
-        <v>56.2</v>
+        <v>0</v>
       </c>
       <c r="S5">
-        <v>43.8</v>
+        <v>100</v>
       </c>
       <c r="T5" t="s">
         <v>151</v>
@@ -2442,13 +2442,13 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>17.2</v>
+        <v>12.5</v>
       </c>
       <c r="Y5">
-        <v>80.09999999999999</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="Z5">
-        <v>61.9</v>
+        <v>55.5</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2466,76 +2466,76 @@
         <v>157</v>
       </c>
       <c r="AF5">
-        <v>85.90000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AG5">
-        <v>91.8</v>
+        <v>94.8</v>
       </c>
       <c r="AH5">
-        <v>71</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AI5">
-        <v>63.6</v>
+        <v>63.5</v>
       </c>
       <c r="AJ5">
-        <v>1010</v>
+        <v>1009.9</v>
       </c>
       <c r="AK5">
-        <v>1012.3</v>
+        <v>1012.1</v>
       </c>
       <c r="AL5">
-        <v>61.6</v>
+        <v>26.4</v>
       </c>
       <c r="AM5">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>31.9</v>
+        <v>32.1</v>
       </c>
       <c r="AP5">
-        <v>2090</v>
+        <v>2709</v>
       </c>
       <c r="AQ5">
-        <v>6.6</v>
+        <v>4.6</v>
       </c>
       <c r="AR5">
-        <v>12.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AS5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AT5">
-        <v>285.7</v>
+        <v>353.1</v>
       </c>
       <c r="AU5">
-        <v>-0.6</v>
+        <v>-4.4</v>
       </c>
       <c r="AV5">
+        <v>-4.4</v>
+      </c>
+      <c r="AW5">
+        <v>-2.8</v>
+      </c>
+      <c r="AX5">
         <v>-4.3</v>
       </c>
-      <c r="AW5">
-        <v>3.2</v>
-      </c>
-      <c r="AX5">
-        <v>-0.6</v>
-      </c>
       <c r="AY5">
+        <v>-3.9</v>
+      </c>
+      <c r="AZ5">
+        <v>-2.6</v>
+      </c>
+      <c r="BA5">
+        <v>1.3</v>
+      </c>
+      <c r="BB5">
         <v>-3.8</v>
       </c>
-      <c r="AZ5">
-        <v>3</v>
-      </c>
-      <c r="BA5">
-        <v>6.4</v>
-      </c>
-      <c r="BB5">
-        <v>-0.5</v>
-      </c>
       <c r="BC5">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="BD5">
         <v>0.9399999999999999</v>
@@ -2550,13 +2550,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.1497</v>
+        <v>1.149</v>
       </c>
       <c r="BI5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BJ5">
-        <v>1883</v>
+        <v>1900</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2565,49 +2565,49 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>64.90000000000001</v>
+        <v>56</v>
       </c>
       <c r="BN5">
-        <v>1.036</v>
+        <v>1.014</v>
       </c>
       <c r="BO5">
-        <v>68.09999999999999</v>
+        <v>57.1</v>
       </c>
       <c r="BP5">
-        <v>61.9</v>
+        <v>56</v>
       </c>
       <c r="BQ5">
-        <v>55.8</v>
+        <v>51</v>
       </c>
       <c r="BR5">
-        <v>54.7</v>
+        <v>53.1</v>
       </c>
       <c r="BS5">
-        <v>52.2</v>
+        <v>51.6</v>
       </c>
       <c r="BT5">
-        <v>20.8</v>
+        <v>16.4</v>
       </c>
       <c r="BU5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BV5">
-        <v>22.2</v>
+        <v>6.9</v>
       </c>
       <c r="BW5" t="s">
         <v>70</v>
       </c>
       <c r="BX5">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="BY5">
-        <v>83.09999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="BZ5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="CA5">
-        <v>4</v>
+        <v>4.4</v>
       </c>
     </row>
   </sheetData>
@@ -2709,34 +2709,34 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>61.9</v>
+        <v>60.1</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>80.8</v>
+        <v>88.2</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I2">
         <v>5</v>
       </c>
       <c r="J2">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L2" t="s">
         <v>67</v>
       </c>
       <c r="M2">
-        <v>90.8</v>
+        <v>91.3</v>
       </c>
       <c r="N2">
-        <v>2253</v>
+        <v>2294</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:05 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="159">
   <si>
     <t>Date</t>
   </si>
@@ -206,37 +206,34 @@
     <t>OPEN-AIR PARK</t>
   </si>
   <si>
-    <t>Partly cloudy</t>
-  </si>
-  <si>
-    <t>🟢 6.8 mph Out to RF</t>
-  </si>
-  <si>
-    <t>W</t>
+    <t>Mostly clear</t>
+  </si>
+  <si>
+    <t>🔴 6.9 mph In from LF</t>
+  </si>
+  <si>
+    <t>WNW</t>
   </si>
   <si>
     <t>FORECAST MODEL</t>
   </si>
   <si>
-    <t>B+</t>
-  </si>
-  <si>
-    <t>Density 87 | Wind 47 | Temp 70 | Altitude 66 | Confidence 88%</t>
-  </si>
-  <si>
-    <t>🟢 Good</t>
-  </si>
-  <si>
-    <t>IMPROVING</t>
-  </si>
-  <si>
-    <t>MODERATE</t>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Density 87 | Wind 41 | Temp 71 | Altitude 66 | Confidence 90%</t>
+  </si>
+  <si>
+    <t>🟨 Neutral</t>
+  </si>
+  <si>
+    <t>STEADY</t>
   </si>
   <si>
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 04:13:23 PM PDT</t>
+    <t>2026-07-16 05:05:47 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -470,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-16 23:13:23 UTC</t>
+    <t>2026-07-17 00:05:47 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -497,10 +494,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>WNW</t>
-  </si>
-  <si>
-    <t>N</t>
+    <t>NW</t>
   </si>
   <si>
     <t>LIGHT</t>
@@ -964,7 +958,7 @@
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="27.7109375" customWidth="1"/>
     <col min="12" max="12" width="33.7109375" customWidth="1"/>
-    <col min="13" max="13" width="21.7109375" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" customWidth="1"/>
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" customWidth="1"/>
@@ -1189,37 +1183,37 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="L2">
-        <v>48.5</v>
+        <v>45.1</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
+        <v>-6.9</v>
+      </c>
+      <c r="Q2">
         <v>-2.6</v>
       </c>
-      <c r="Q2">
-        <v>2.6</v>
-      </c>
       <c r="R2">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
       </c>
       <c r="U2">
-        <v>22.4</v>
+        <v>11.8</v>
       </c>
       <c r="V2">
-        <v>60.1</v>
+        <v>58.6</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1228,25 +1222,25 @@
         <v>66</v>
       </c>
       <c r="Y2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Z2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA2">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="AB2">
-        <v>88.2</v>
+        <v>89.5</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>-1.2</v>
+        <v>-3.2</v>
       </c>
       <c r="AE2">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="AF2">
         <v>22.5</v>
@@ -1255,34 +1249,34 @@
         <v>77.5</v>
       </c>
       <c r="AH2">
-        <v>29.5</v>
+        <v>11.1</v>
       </c>
       <c r="AI2">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="AJ2">
-        <v>1.1367</v>
+        <v>1.1365</v>
       </c>
       <c r="AK2">
-        <v>2294</v>
+        <v>2327</v>
       </c>
       <c r="AL2">
-        <v>1008.5</v>
+        <v>1008.4</v>
       </c>
       <c r="AM2">
-        <v>70.90000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AN2">
-        <v>91.3</v>
+        <v>91.8</v>
       </c>
       <c r="AO2">
-        <v>52.8</v>
+        <v>48.1</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>3</v>
+        <v>-0.9</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1294,19 +1288,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>24.3</v>
+        <v>19.3</v>
       </c>
       <c r="AV2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AW2">
+        <v>12.2</v>
+      </c>
+      <c r="AX2" t="s">
         <v>70</v>
       </c>
-      <c r="AW2">
-        <v>17.9</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>71</v>
-      </c>
       <c r="AY2">
-        <v>184.5</v>
+        <v>236.9</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1374,7 +1368,7 @@
     <col min="28" max="28" width="27.7109375" customWidth="1"/>
     <col min="29" max="29" width="17.7109375" customWidth="1"/>
     <col min="30" max="30" width="25.7109375" customWidth="1"/>
-    <col min="31" max="31" width="15.7109375" customWidth="1"/>
+    <col min="31" max="31" width="14.7109375" customWidth="1"/>
     <col min="32" max="32" width="10.7109375" customWidth="1"/>
     <col min="33" max="33" width="14.7109375" customWidth="1"/>
     <col min="34" max="34" width="13.7109375" customWidth="1"/>
@@ -1429,211 +1423,211 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="BV1" s="1" t="s">
         <v>48</v>
@@ -1642,16 +1636,16 @@
         <v>47</v>
       </c>
       <c r="BX1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:79">
@@ -1668,22 +1662,22 @@
         <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F2" t="s">
         <v>57</v>
       </c>
       <c r="G2" t="s">
+        <v>148</v>
+      </c>
+      <c r="H2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I2" t="s">
         <v>149</v>
       </c>
-      <c r="H2" t="s">
-        <v>71</v>
-      </c>
-      <c r="I2" t="s">
-        <v>150</v>
-      </c>
       <c r="J2">
-        <v>184.5</v>
+        <v>236.9</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1692,19 +1686,19 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.11</v>
+        <v>2.44</v>
       </c>
       <c r="N2">
-        <v>0.09</v>
+        <v>1.22</v>
       </c>
       <c r="O2">
         <v>9.33</v>
       </c>
       <c r="P2">
-        <v>32.6</v>
+        <v>11.9</v>
       </c>
       <c r="Q2">
-        <v>3.8</v>
+        <v>1.7</v>
       </c>
       <c r="R2">
         <v>56.2</v>
@@ -1713,25 +1707,25 @@
         <v>43.8</v>
       </c>
       <c r="T2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U2" t="s">
         <v>151</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>152</v>
-      </c>
-      <c r="V2" t="s">
-        <v>153</v>
       </c>
       <c r="W2">
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>8</v>
+        <v>16.7</v>
       </c>
       <c r="Y2">
-        <v>93.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="Z2">
-        <v>76.2</v>
+        <v>61.7</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1749,76 +1743,76 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="AG2">
-        <v>99.40000000000001</v>
+        <v>101.2</v>
       </c>
       <c r="AH2">
-        <v>70.90000000000001</v>
+        <v>68.8</v>
       </c>
       <c r="AI2">
-        <v>48.5</v>
+        <v>45.1</v>
       </c>
       <c r="AJ2">
-        <v>1008</v>
+        <v>1007.8</v>
       </c>
       <c r="AK2">
-        <v>1010.2</v>
+        <v>1010</v>
       </c>
       <c r="AL2">
-        <v>72.5</v>
+        <v>36.9</v>
       </c>
       <c r="AM2">
-        <v>22.4</v>
+        <v>11.8</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>60.2</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="AP2">
-        <v>2705</v>
+        <v>1791</v>
       </c>
       <c r="AQ2">
-        <v>9.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="AR2">
-        <v>17.7</v>
+        <v>22.4</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>263.1</v>
+        <v>295.4</v>
       </c>
       <c r="AU2">
-        <v>2.7</v>
+        <v>-2.7</v>
       </c>
       <c r="AV2">
-        <v>-2.9</v>
+        <v>-7.7</v>
       </c>
       <c r="AW2">
-        <v>7.3</v>
+        <v>3.4</v>
       </c>
       <c r="AX2">
-        <v>2.6</v>
+        <v>-2.6</v>
       </c>
       <c r="AY2">
-        <v>-2.6</v>
+        <v>-6.9</v>
       </c>
       <c r="AZ2">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
       <c r="BA2">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="BB2">
-        <v>2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="BC2">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="BD2">
         <v>0.9399999999999999</v>
@@ -1833,13 +1827,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1309</v>
+        <v>1.1312</v>
       </c>
       <c r="BI2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="BJ2">
-        <v>2476</v>
+        <v>2493</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1848,49 +1842,49 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>78</v>
+        <v>63.6</v>
       </c>
       <c r="BN2">
-        <v>1.067</v>
+        <v>1.033</v>
       </c>
       <c r="BO2">
-        <v>81.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="BP2">
-        <v>73.5</v>
+        <v>59.4</v>
       </c>
       <c r="BQ2">
-        <v>60.6</v>
+        <v>58</v>
       </c>
       <c r="BR2">
-        <v>57.9</v>
+        <v>55.3</v>
       </c>
       <c r="BS2">
-        <v>41.3</v>
+        <v>39.3</v>
       </c>
       <c r="BT2">
-        <v>24.3</v>
+        <v>18.5</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>5.1</v>
+        <v>12.2</v>
       </c>
       <c r="BW2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BX2">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="BY2">
-        <v>92.5</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="BZ2">
         <v>10</v>
       </c>
       <c r="CA2">
-        <v>9</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1907,22 +1901,22 @@
         <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" t="s">
         <v>149</v>
       </c>
-      <c r="H3" t="s">
-        <v>71</v>
-      </c>
-      <c r="I3" t="s">
-        <v>150</v>
-      </c>
       <c r="J3">
-        <v>184.5</v>
+        <v>236.9</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -1931,19 +1925,19 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.77</v>
+        <v>1.19</v>
       </c>
       <c r="N3">
-        <v>2.84</v>
+        <v>0.39</v>
       </c>
       <c r="O3">
-        <v>7.53</v>
+        <v>7.49</v>
       </c>
       <c r="P3">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="Q3">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -1952,25 +1946,25 @@
         <v>100</v>
       </c>
       <c r="T3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="U3" t="s">
+        <v>152</v>
+      </c>
+      <c r="V3" t="s">
         <v>153</v>
-      </c>
-      <c r="V3" t="s">
-        <v>154</v>
       </c>
       <c r="W3">
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>18.2</v>
+        <v>8.6</v>
       </c>
       <c r="Y3">
-        <v>83.40000000000001</v>
+        <v>92.3</v>
       </c>
       <c r="Z3">
-        <v>61</v>
+        <v>59.6</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1985,79 +1979,79 @@
         <v>1.6</v>
       </c>
       <c r="AE3" t="s">
-        <v>61</v>
+        <v>156</v>
       </c>
       <c r="AF3">
-        <v>91.3</v>
+        <v>91.7</v>
       </c>
       <c r="AG3">
-        <v>98.3</v>
+        <v>96.8</v>
       </c>
       <c r="AH3">
-        <v>70.5</v>
+        <v>68.7</v>
       </c>
       <c r="AI3">
-        <v>51.9</v>
+        <v>48.3</v>
       </c>
       <c r="AJ3">
         <v>1008.3</v>
       </c>
       <c r="AK3">
-        <v>1010.6</v>
+        <v>1010.5</v>
       </c>
       <c r="AL3">
-        <v>61.9</v>
+        <v>25.1</v>
       </c>
       <c r="AM3">
-        <v>17.4</v>
+        <v>13.3</v>
       </c>
       <c r="AN3">
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>53.7</v>
+        <v>62.5</v>
       </c>
       <c r="AP3">
-        <v>2300</v>
+        <v>1689</v>
       </c>
       <c r="AQ3">
-        <v>7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AR3">
-        <v>13.1</v>
+        <v>18.5</v>
       </c>
       <c r="AS3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AT3">
-        <v>302.1</v>
+        <v>304.6</v>
       </c>
       <c r="AU3">
-        <v>-2.6</v>
+        <v>-3.6</v>
       </c>
       <c r="AV3">
-        <v>-5.9</v>
+        <v>-7.6</v>
       </c>
       <c r="AW3">
         <v>1.6</v>
       </c>
       <c r="AX3">
-        <v>-2.6</v>
+        <v>-3.6</v>
       </c>
       <c r="AY3">
-        <v>-5.2</v>
+        <v>-6.8</v>
       </c>
       <c r="AZ3">
         <v>1.5</v>
       </c>
       <c r="BA3">
-        <v>6.3</v>
+        <v>7.8</v>
       </c>
       <c r="BB3">
-        <v>-2.3</v>
+        <v>-3.2</v>
       </c>
       <c r="BC3">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BD3">
         <v>0.9399999999999999</v>
@@ -2072,13 +2066,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1366</v>
+        <v>1.1365</v>
       </c>
       <c r="BI3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="BJ3">
-        <v>2301</v>
+        <v>2325</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2087,49 +2081,49 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>63.2</v>
+        <v>60.4</v>
       </c>
       <c r="BN3">
-        <v>1.032</v>
+        <v>1.025</v>
       </c>
       <c r="BO3">
-        <v>66.59999999999999</v>
+        <v>64.5</v>
       </c>
       <c r="BP3">
-        <v>60.5</v>
+        <v>57.1</v>
       </c>
       <c r="BQ3">
-        <v>55.8</v>
+        <v>56</v>
       </c>
       <c r="BR3">
-        <v>55</v>
+        <v>54.4</v>
       </c>
       <c r="BS3">
-        <v>46.6</v>
+        <v>45.1</v>
       </c>
       <c r="BT3">
-        <v>21.6</v>
+        <v>19.3</v>
       </c>
       <c r="BU3" t="s">
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>15.2</v>
+        <v>7.1</v>
       </c>
       <c r="BW3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BX3">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="BY3">
-        <v>89.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>4.8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2146,43 +2140,43 @@
         <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G4" t="s">
+        <v>148</v>
+      </c>
+      <c r="H4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I4" t="s">
         <v>149</v>
       </c>
-      <c r="H4" t="s">
-        <v>71</v>
-      </c>
-      <c r="I4" t="s">
-        <v>150</v>
-      </c>
       <c r="J4">
-        <v>184.5</v>
+        <v>236.9</v>
       </c>
       <c r="K4">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.61</v>
+        <v>0.97</v>
       </c>
       <c r="N4">
-        <v>2.15</v>
+        <v>0.52</v>
       </c>
       <c r="O4">
-        <v>6.66</v>
+        <v>6.68</v>
       </c>
       <c r="P4">
-        <v>46</v>
+        <v>5.9</v>
       </c>
       <c r="Q4">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -2191,25 +2185,25 @@
         <v>100</v>
       </c>
       <c r="T4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="U4" t="s">
+        <v>153</v>
+      </c>
+      <c r="V4" t="s">
         <v>154</v>
-      </c>
-      <c r="V4" t="s">
-        <v>155</v>
       </c>
       <c r="W4">
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>15.2</v>
+        <v>7.8</v>
       </c>
       <c r="Y4">
-        <v>83.3</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Z4">
-        <v>52.7</v>
+        <v>54.9</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2224,79 +2218,79 @@
         <v>1.6</v>
       </c>
       <c r="AE4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF4">
-        <v>89</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AG4">
-        <v>97.2</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="AH4">
-        <v>71.2</v>
+        <v>69</v>
       </c>
       <c r="AI4">
-        <v>57.4</v>
+        <v>51.5</v>
       </c>
       <c r="AJ4">
-        <v>1009.2</v>
+        <v>1009</v>
       </c>
       <c r="AK4">
-        <v>1011.5</v>
+        <v>1011.3</v>
       </c>
       <c r="AL4">
-        <v>20</v>
+        <v>23.3</v>
       </c>
       <c r="AM4">
-        <v>10.6</v>
+        <v>10.1</v>
       </c>
       <c r="AN4">
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>43.7</v>
+        <v>42</v>
       </c>
       <c r="AP4">
-        <v>2571</v>
+        <v>1744</v>
       </c>
       <c r="AQ4">
-        <v>6.6</v>
+        <v>8.1</v>
       </c>
       <c r="AR4">
-        <v>9.4</v>
+        <v>14.4</v>
       </c>
       <c r="AS4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="AT4">
-        <v>352</v>
+        <v>322</v>
       </c>
       <c r="AU4">
-        <v>-6.2</v>
+        <v>-5.4</v>
       </c>
       <c r="AV4">
-        <v>-6.3</v>
+        <v>-7.9</v>
       </c>
       <c r="AW4">
-        <v>-3.9</v>
+        <v>-1</v>
       </c>
       <c r="AX4">
-        <v>-6.1</v>
+        <v>-5.3</v>
       </c>
       <c r="AY4">
-        <v>-5.6</v>
+        <v>-7.1</v>
       </c>
       <c r="AZ4">
-        <v>-3.7</v>
+        <v>-0.9</v>
       </c>
       <c r="BA4">
-        <v>2</v>
+        <v>5.9</v>
       </c>
       <c r="BB4">
-        <v>-5.5</v>
+        <v>-4.7</v>
       </c>
       <c r="BC4">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="BD4">
         <v>0.9399999999999999</v>
@@ -2311,13 +2305,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1421</v>
+        <v>1.1408</v>
       </c>
       <c r="BI4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="BJ4">
-        <v>2117</v>
+        <v>2184</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2326,49 +2320,49 @@
         <v>60</v>
       </c>
       <c r="BM4">
+        <v>55.4</v>
+      </c>
+      <c r="BN4">
+        <v>1.013</v>
+      </c>
+      <c r="BO4">
+        <v>58.8</v>
+      </c>
+      <c r="BP4">
         <v>53.3</v>
       </c>
-      <c r="BN4">
-        <v>1.008</v>
-      </c>
-      <c r="BO4">
-        <v>54.9</v>
-      </c>
-      <c r="BP4">
-        <v>53.1</v>
-      </c>
       <c r="BQ4">
-        <v>50.9</v>
+        <v>53.6</v>
       </c>
       <c r="BR4">
-        <v>53</v>
+        <v>53.3</v>
       </c>
       <c r="BS4">
-        <v>48.5</v>
+        <v>49.5</v>
       </c>
       <c r="BT4">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="BU4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BV4">
-        <v>17.9</v>
+        <v>9</v>
       </c>
       <c r="BW4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BX4">
         <v>90</v>
       </c>
       <c r="BY4">
-        <v>87.09999999999999</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>4</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2385,43 +2379,43 @@
         <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F5" t="s">
+        <v>147</v>
+      </c>
+      <c r="G5" t="s">
         <v>148</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I5" t="s">
         <v>149</v>
       </c>
-      <c r="H5" t="s">
-        <v>71</v>
-      </c>
-      <c r="I5" t="s">
-        <v>150</v>
-      </c>
       <c r="J5">
-        <v>184.5</v>
+        <v>236.9</v>
       </c>
       <c r="K5">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.67</v>
+        <v>0.96</v>
       </c>
       <c r="N5">
-        <v>1.43</v>
+        <v>1.35</v>
       </c>
       <c r="O5">
         <v>4.26</v>
       </c>
       <c r="P5">
-        <v>37</v>
+        <v>10.6</v>
       </c>
       <c r="Q5">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -2430,25 +2424,25 @@
         <v>100</v>
       </c>
       <c r="T5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="U5" t="s">
+        <v>154</v>
+      </c>
+      <c r="V5" t="s">
         <v>155</v>
-      </c>
-      <c r="V5" t="s">
-        <v>156</v>
       </c>
       <c r="W5">
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>12.5</v>
+        <v>9.4</v>
       </c>
       <c r="Y5">
-        <v>90.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="Z5">
-        <v>55.5</v>
+        <v>56.3</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2463,28 +2457,28 @@
         <v>1.6</v>
       </c>
       <c r="AE5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AF5">
-        <v>86.09999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="AG5">
-        <v>94.8</v>
+        <v>87.8</v>
       </c>
       <c r="AH5">
-        <v>71.40000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="AI5">
-        <v>63.5</v>
+        <v>52.6</v>
       </c>
       <c r="AJ5">
-        <v>1009.9</v>
+        <v>1009.6</v>
       </c>
       <c r="AK5">
-        <v>1012.1</v>
+        <v>1011.9</v>
       </c>
       <c r="AL5">
-        <v>26.4</v>
+        <v>25</v>
       </c>
       <c r="AM5">
         <v>8</v>
@@ -2493,49 +2487,49 @@
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>32.1</v>
+        <v>38.7</v>
       </c>
       <c r="AP5">
-        <v>2709</v>
+        <v>592</v>
       </c>
       <c r="AQ5">
-        <v>4.6</v>
+        <v>6</v>
       </c>
       <c r="AR5">
-        <v>8.199999999999999</v>
+        <v>13.4</v>
       </c>
       <c r="AS5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="AT5">
-        <v>353.1</v>
+        <v>322.2</v>
       </c>
       <c r="AU5">
-        <v>-4.4</v>
+        <v>-4</v>
       </c>
       <c r="AV5">
-        <v>-4.4</v>
+        <v>-5.9</v>
       </c>
       <c r="AW5">
-        <v>-2.8</v>
+        <v>-0.8</v>
       </c>
       <c r="AX5">
-        <v>-4.3</v>
+        <v>-3.9</v>
       </c>
       <c r="AY5">
-        <v>-3.9</v>
+        <v>-5.2</v>
       </c>
       <c r="AZ5">
-        <v>-2.6</v>
+        <v>-0.7</v>
       </c>
       <c r="BA5">
-        <v>1.3</v>
+        <v>4.4</v>
       </c>
       <c r="BB5">
-        <v>-3.8</v>
+        <v>-3.5</v>
       </c>
       <c r="BC5">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="BD5">
         <v>0.9399999999999999</v>
@@ -2553,10 +2547,10 @@
         <v>1.149</v>
       </c>
       <c r="BI5" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="BJ5">
-        <v>1900</v>
+        <v>1954</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2565,49 +2559,49 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>56</v>
+        <v>56.9</v>
       </c>
       <c r="BN5">
-        <v>1.014</v>
+        <v>1.017</v>
       </c>
       <c r="BO5">
-        <v>57.1</v>
+        <v>59.4</v>
       </c>
       <c r="BP5">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="BQ5">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="BR5">
-        <v>53.1</v>
+        <v>52.9</v>
       </c>
       <c r="BS5">
-        <v>51.6</v>
+        <v>55.2</v>
       </c>
       <c r="BT5">
-        <v>16.4</v>
+        <v>10.3</v>
       </c>
       <c r="BU5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BV5">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="BW5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BX5">
         <v>87</v>
       </c>
       <c r="BY5">
-        <v>84.2</v>
+        <v>85.3</v>
       </c>
       <c r="BZ5">
         <v>5</v>
       </c>
       <c r="CA5">
-        <v>4.4</v>
+        <v>7.1</v>
       </c>
     </row>
   </sheetData>
@@ -2709,34 +2703,34 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>60.1</v>
+        <v>58.6</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>88.2</v>
+        <v>89.5</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="K2">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="L2" t="s">
         <v>67</v>
       </c>
       <c r="M2">
-        <v>91.3</v>
+        <v>91.8</v>
       </c>
       <c r="N2">
-        <v>2294</v>
+        <v>2327</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:09 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:05:47 PM PDT</t>
+    <t>2026-07-16 05:09:12 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:05:47 UTC</t>
+    <t>2026-07-17 00:09:12 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1276,7 +1276,7 @@
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>-0.9</v>
+        <v>0.6</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>236.9</v>
+        <v>240.4</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>236.9</v>
+        <v>240.4</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>236.9</v>
+        <v>240.4</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,10 +2155,10 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>236.9</v>
+        <v>240.4</v>
       </c>
       <c r="K4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -2394,10 +2394,10 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>236.9</v>
+        <v>240.4</v>
       </c>
       <c r="K5">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="L5">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:13 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:09:24 PM PDT</t>
+    <t>2026-07-16 05:13:36 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:09:24 UTC</t>
+    <t>2026-07-17 00:13:36 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>240.6</v>
+        <v>244.8</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>240.6</v>
+        <v>244.8</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>240.6</v>
+        <v>244.8</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>240.6</v>
+        <v>244.8</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,10 +2394,10 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>240.6</v>
+        <v>244.8</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L5">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:14 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:13:36 PM PDT</t>
+    <t>2026-07-16 05:14:12 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:13:36 UTC</t>
+    <t>2026-07-17 00:14:12 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>244.8</v>
+        <v>245.4</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>244.8</v>
+        <v>245.4</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>244.8</v>
+        <v>245.4</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>244.8</v>
+        <v>245.4</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,7 +2394,7 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>244.8</v>
+        <v>245.4</v>
       </c>
       <c r="K5">
         <v>0.9</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:18 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:14:46 PM PDT</t>
+    <t>2026-07-16 05:18:50 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:14:46 UTC</t>
+    <t>2026-07-17 00:18:50 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1276,7 +1276,7 @@
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>245.9</v>
+        <v>250</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>245.9</v>
+        <v>250</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>245.9</v>
+        <v>250</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>245.9</v>
+        <v>250</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,7 +2394,7 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>245.9</v>
+        <v>250</v>
       </c>
       <c r="K5">
         <v>0.9</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:19 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:18:50 PM PDT</t>
+    <t>2026-07-16 05:19:10 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:18:50 UTC</t>
+    <t>2026-07-17 00:19:10 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>250</v>
+        <v>250.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>250</v>
+        <v>250.3</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>250</v>
+        <v>250.3</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>250</v>
+        <v>250.3</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,10 +2394,10 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>250</v>
+        <v>250.3</v>
       </c>
       <c r="K5">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L5">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:20 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:19:10 PM PDT</t>
+    <t>2026-07-16 05:20:20 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:19:10 UTC</t>
+    <t>2026-07-17 00:20:20 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>250.3</v>
+        <v>251.5</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>250.3</v>
+        <v>251.5</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>250.3</v>
+        <v>251.5</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>250.3</v>
+        <v>251.5</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,7 +2394,7 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>250.3</v>
+        <v>251.5</v>
       </c>
       <c r="K5">
         <v>0.8</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:22 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:20:20 PM PDT</t>
+    <t>2026-07-16 05:22:01 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:20:20 UTC</t>
+    <t>2026-07-17 00:22:01 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -1300,7 +1300,7 @@
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>251.5</v>
+        <v>253.2</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>251.5</v>
+        <v>253.2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>251.5</v>
+        <v>253.2</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>251.5</v>
+        <v>253.2</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2394,7 +2394,7 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>251.5</v>
+        <v>253.2</v>
       </c>
       <c r="K5">
         <v>0.8</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-16 05:43 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_16.xlsx
+++ b/mlb_weather_professional_v4_2026_07_16.xlsx
@@ -209,7 +209,7 @@
     <t>Mostly clear</t>
   </si>
   <si>
-    <t>🟡 3.1 mph Cross (LF → RF)</t>
+    <t>🟡 3.2 mph Cross (LF → RF)</t>
   </si>
   <si>
     <t>WNW</t>
@@ -221,7 +221,7 @@
     <t>B</t>
   </si>
   <si>
-    <t>Density 87 | Wind 41 | Temp 71 | Altitude 66 | Confidence 90%</t>
+    <t>Density 88 | Wind 42 | Temp 71 | Altitude 66 | Confidence 88%</t>
   </si>
   <si>
     <t>🟨 Neutral</t>
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-16 05:22:51 PM PDT</t>
+    <t>2026-07-16 05:43:11 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>09:10 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-17 00:22:51 UTC</t>
+    <t>2026-07-17 00:43:11 UTC</t>
   </si>
   <si>
     <t>2026-07-16T20:08:51+00:00</t>
@@ -491,7 +491,7 @@
     <t>2026-07-16T22:00</t>
   </si>
   <si>
-    <t>Clear</t>
+    <t>Partly cloudy</t>
   </si>
   <si>
     <t>NW</t>
@@ -1183,37 +1183,37 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>94</v>
+        <v>94.2</v>
       </c>
       <c r="L2">
-        <v>45.1</v>
+        <v>44.7</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>10</v>
+        <v>10.2</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>-6.9</v>
+        <v>-7</v>
       </c>
       <c r="Q2">
         <v>-2.6</v>
       </c>
       <c r="R2">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
       </c>
       <c r="U2">
-        <v>11.8</v>
+        <v>10.9</v>
       </c>
       <c r="V2">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1228,16 +1228,16 @@
         <v>4</v>
       </c>
       <c r="AA2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="AB2">
-        <v>89.5</v>
+        <v>87.8</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>-3.2</v>
+        <v>-3</v>
       </c>
       <c r="AE2">
         <v>-3</v>
@@ -1246,37 +1246,37 @@
         <v>22.5</v>
       </c>
       <c r="AG2">
-        <v>77.5</v>
+        <v>60.7</v>
       </c>
       <c r="AH2">
-        <v>11.1</v>
+        <v>12.8</v>
       </c>
       <c r="AI2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1365</v>
+        <v>1.1355</v>
       </c>
       <c r="AK2">
-        <v>2327</v>
+        <v>2366</v>
       </c>
       <c r="AL2">
-        <v>1008.4</v>
+        <v>1008.5</v>
       </c>
       <c r="AM2">
-        <v>68.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="AN2">
-        <v>91.8</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="AO2">
-        <v>48.1</v>
+        <v>46</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1288,19 +1288,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>19.3</v>
+        <v>18.9</v>
       </c>
       <c r="AV2" t="s">
         <v>69</v>
       </c>
       <c r="AW2">
-        <v>12.2</v>
+        <v>13.5</v>
       </c>
       <c r="AX2" t="s">
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>254</v>
+        <v>274.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1368,7 +1368,7 @@
     <col min="28" max="28" width="27.7109375" customWidth="1"/>
     <col min="29" max="29" width="17.7109375" customWidth="1"/>
     <col min="30" max="30" width="25.7109375" customWidth="1"/>
-    <col min="31" max="31" width="14.7109375" customWidth="1"/>
+    <col min="31" max="31" width="15.7109375" customWidth="1"/>
     <col min="32" max="32" width="10.7109375" customWidth="1"/>
     <col min="33" max="33" width="14.7109375" customWidth="1"/>
     <col min="34" max="34" width="13.7109375" customWidth="1"/>
@@ -1677,7 +1677,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>254</v>
+        <v>274.3</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1686,19 +1686,19 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>2.44</v>
+        <v>2.79</v>
       </c>
       <c r="N2">
-        <v>1.22</v>
+        <v>1.43</v>
       </c>
       <c r="O2">
-        <v>9.33</v>
+        <v>6.78</v>
       </c>
       <c r="P2">
-        <v>11.9</v>
+        <v>12.3</v>
       </c>
       <c r="Q2">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="R2">
         <v>56.2</v>
@@ -1719,13 +1719,13 @@
         <v>0.1667</v>
       </c>
       <c r="X2">
-        <v>16.7</v>
+        <v>17.8</v>
       </c>
       <c r="Y2">
-        <v>85.8</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="Z2">
-        <v>61.7</v>
+        <v>61.6</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1743,16 +1743,16 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>94</v>
+        <v>94.2</v>
       </c>
       <c r="AG2">
-        <v>101.2</v>
+        <v>101.5</v>
       </c>
       <c r="AH2">
-        <v>68.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AI2">
-        <v>45.1</v>
+        <v>44.7</v>
       </c>
       <c r="AJ2">
         <v>1007.8</v>
@@ -1761,52 +1761,52 @@
         <v>1010</v>
       </c>
       <c r="AL2">
-        <v>36.9</v>
+        <v>38</v>
       </c>
       <c r="AM2">
-        <v>11.8</v>
+        <v>10.9</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>91.59999999999999</v>
+        <v>97</v>
       </c>
       <c r="AP2">
-        <v>1791</v>
+        <v>1773</v>
       </c>
       <c r="AQ2">
-        <v>10</v>
+        <v>10.2</v>
       </c>
       <c r="AR2">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>295.4</v>
+        <v>295.1</v>
       </c>
       <c r="AU2">
-        <v>-2.7</v>
+        <v>-2.6</v>
       </c>
       <c r="AV2">
-        <v>-7.7</v>
+        <v>-7.8</v>
       </c>
       <c r="AW2">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="AX2">
         <v>-2.6</v>
       </c>
       <c r="AY2">
-        <v>-6.9</v>
+        <v>-7</v>
       </c>
       <c r="AZ2">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="BA2">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="BB2">
         <v>-2.3</v>
@@ -1827,13 +1827,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1312</v>
+        <v>1.1307</v>
       </c>
       <c r="BI2" t="s">
         <v>158</v>
       </c>
       <c r="BJ2">
-        <v>2493</v>
+        <v>2508</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1842,34 +1842,34 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>63.6</v>
+        <v>63.7</v>
       </c>
       <c r="BN2">
         <v>1.033</v>
       </c>
       <c r="BO2">
-        <v>68.5</v>
+        <v>68.7</v>
       </c>
       <c r="BP2">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="BQ2">
-        <v>58</v>
+        <v>58.1</v>
       </c>
       <c r="BR2">
-        <v>55.3</v>
+        <v>55.4</v>
       </c>
       <c r="BS2">
-        <v>39.3</v>
+        <v>39.1</v>
       </c>
       <c r="BT2">
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>12.2</v>
+        <v>13.5</v>
       </c>
       <c r="BW2" t="s">
         <v>69</v>
@@ -1878,13 +1878,13 @@
         <v>90</v>
       </c>
       <c r="BY2">
-        <v>95.59999999999999</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="BZ2">
         <v>10</v>
       </c>
       <c r="CA2">
-        <v>10.5</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1916,7 +1916,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>254</v>
+        <v>274.3</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -1925,25 +1925,25 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.19</v>
+        <v>2.69</v>
       </c>
       <c r="N3">
-        <v>0.39</v>
+        <v>1.27</v>
       </c>
       <c r="O3">
-        <v>7.49</v>
+        <v>6.05</v>
       </c>
       <c r="P3">
-        <v>13.5</v>
+        <v>17.4</v>
       </c>
       <c r="Q3">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="R3">
         <v>0</v>
       </c>
       <c r="S3">
-        <v>100</v>
+        <v>43.8</v>
       </c>
       <c r="T3" t="s">
         <v>150</v>
@@ -1958,13 +1958,13 @@
         <v>0.1667</v>
       </c>
       <c r="X3">
-        <v>8.6</v>
+        <v>16.7</v>
       </c>
       <c r="Y3">
-        <v>92.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="Z3">
-        <v>59.6</v>
+        <v>59.8</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1979,76 +1979,76 @@
         <v>1.6</v>
       </c>
       <c r="AE3" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="AF3">
-        <v>91.7</v>
+        <v>93</v>
       </c>
       <c r="AG3">
-        <v>96.8</v>
+        <v>98.5</v>
       </c>
       <c r="AH3">
-        <v>68.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="AI3">
-        <v>48.3</v>
+        <v>45</v>
       </c>
       <c r="AJ3">
-        <v>1008.3</v>
+        <v>1008.4</v>
       </c>
       <c r="AK3">
-        <v>1010.5</v>
+        <v>1010.7</v>
       </c>
       <c r="AL3">
-        <v>25.1</v>
+        <v>32.1</v>
       </c>
       <c r="AM3">
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="AN3">
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>62.5</v>
+        <v>87.8</v>
       </c>
       <c r="AP3">
-        <v>1689</v>
+        <v>1434</v>
       </c>
       <c r="AQ3">
-        <v>8.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="AR3">
-        <v>18.5</v>
+        <v>19.1</v>
       </c>
       <c r="AS3" t="s">
-        <v>157</v>
+        <v>63</v>
       </c>
       <c r="AT3">
-        <v>304.6</v>
+        <v>301.9</v>
       </c>
       <c r="AU3">
-        <v>-3.6</v>
+        <v>-3.5</v>
       </c>
       <c r="AV3">
-        <v>-7.6</v>
+        <v>-7.9</v>
       </c>
       <c r="AW3">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="AX3">
-        <v>-3.6</v>
+        <v>-3.4</v>
       </c>
       <c r="AY3">
-        <v>-6.8</v>
+        <v>-7</v>
       </c>
       <c r="AZ3">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="BA3">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="BB3">
-        <v>-3.2</v>
+        <v>-3</v>
       </c>
       <c r="BC3">
         <v>0.8</v>
@@ -2066,13 +2066,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1365</v>
+        <v>1.1343</v>
       </c>
       <c r="BI3" t="s">
         <v>158</v>
       </c>
       <c r="BJ3">
-        <v>2325</v>
+        <v>2407</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2081,34 +2081,34 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>60.4</v>
+        <v>61.2</v>
       </c>
       <c r="BN3">
-        <v>1.025</v>
+        <v>1.027</v>
       </c>
       <c r="BO3">
-        <v>64.5</v>
+        <v>65.7</v>
       </c>
       <c r="BP3">
-        <v>57.1</v>
+        <v>57.6</v>
       </c>
       <c r="BQ3">
-        <v>56</v>
+        <v>56.8</v>
       </c>
       <c r="BR3">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="BS3">
-        <v>45.1</v>
+        <v>44.2</v>
       </c>
       <c r="BT3">
-        <v>19.3</v>
+        <v>18.9</v>
       </c>
       <c r="BU3" t="s">
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>7.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BW3" t="s">
         <v>69</v>
@@ -2117,13 +2117,13 @@
         <v>90</v>
       </c>
       <c r="BY3">
-        <v>91.7</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>8.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2155,7 +2155,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>254</v>
+        <v>274.3</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2164,19 +2164,19 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>0.97</v>
+        <v>1.41</v>
       </c>
       <c r="N4">
-        <v>0.52</v>
+        <v>0.32</v>
       </c>
       <c r="O4">
-        <v>6.68</v>
+        <v>5.38</v>
       </c>
       <c r="P4">
-        <v>5.9</v>
+        <v>10.3</v>
       </c>
       <c r="Q4">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -2197,13 +2197,13 @@
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>7.8</v>
+        <v>8.5</v>
       </c>
       <c r="Y4">
-        <v>91.59999999999999</v>
+        <v>92</v>
       </c>
       <c r="Z4">
-        <v>54.9</v>
+        <v>56.7</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2218,76 +2218,76 @@
         <v>1.6</v>
       </c>
       <c r="AE4" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="AF4">
-        <v>89.90000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="AG4">
-        <v>94.40000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="AH4">
-        <v>69</v>
+        <v>66.8</v>
       </c>
       <c r="AI4">
-        <v>51.5</v>
+        <v>47.5</v>
       </c>
       <c r="AJ4">
-        <v>1009</v>
+        <v>1009.2</v>
       </c>
       <c r="AK4">
-        <v>1011.3</v>
+        <v>1011.4</v>
       </c>
       <c r="AL4">
-        <v>23.3</v>
+        <v>39</v>
       </c>
       <c r="AM4">
-        <v>10.1</v>
+        <v>9.6</v>
       </c>
       <c r="AN4">
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>42</v>
+        <v>32.3</v>
       </c>
       <c r="AP4">
-        <v>1744</v>
+        <v>891</v>
       </c>
       <c r="AQ4">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="AR4">
-        <v>14.4</v>
+        <v>13.9</v>
       </c>
       <c r="AS4" t="s">
         <v>157</v>
       </c>
       <c r="AT4">
-        <v>322</v>
+        <v>316.4</v>
       </c>
       <c r="AU4">
-        <v>-5.4</v>
+        <v>-4.7</v>
       </c>
       <c r="AV4">
-        <v>-7.9</v>
+        <v>-7.5</v>
       </c>
       <c r="AW4">
-        <v>-1</v>
+        <v>-0.2</v>
       </c>
       <c r="AX4">
-        <v>-5.3</v>
+        <v>-4.6</v>
       </c>
       <c r="AY4">
-        <v>-7.1</v>
+        <v>-6.7</v>
       </c>
       <c r="AZ4">
-        <v>-0.9</v>
+        <v>-0.2</v>
       </c>
       <c r="BA4">
-        <v>5.9</v>
+        <v>6.3</v>
       </c>
       <c r="BB4">
-        <v>-4.7</v>
+        <v>-4.1</v>
       </c>
       <c r="BC4">
         <v>0.7</v>
@@ -2305,13 +2305,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1408</v>
+        <v>1.1405</v>
       </c>
       <c r="BI4" t="s">
         <v>158</v>
       </c>
       <c r="BJ4">
-        <v>2184</v>
+        <v>2219</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2320,34 +2320,34 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>55.4</v>
+        <v>57.3</v>
       </c>
       <c r="BN4">
-        <v>1.013</v>
+        <v>1.018</v>
       </c>
       <c r="BO4">
-        <v>58.8</v>
+        <v>60.8</v>
       </c>
       <c r="BP4">
-        <v>53.3</v>
+        <v>54.9</v>
       </c>
       <c r="BQ4">
-        <v>53.6</v>
+        <v>54.4</v>
       </c>
       <c r="BR4">
-        <v>53.3</v>
+        <v>53.5</v>
       </c>
       <c r="BS4">
-        <v>49.5</v>
+        <v>50.8</v>
       </c>
       <c r="BT4">
-        <v>17.6</v>
+        <v>14.2</v>
       </c>
       <c r="BU4" t="s">
         <v>69</v>
       </c>
       <c r="BV4">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="BW4" t="s">
         <v>69</v>
@@ -2356,13 +2356,13 @@
         <v>90</v>
       </c>
       <c r="BY4">
-        <v>88.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2394,25 +2394,25 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>254</v>
+        <v>274.3</v>
       </c>
       <c r="K5">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.96</v>
+        <v>0.89</v>
       </c>
       <c r="N5">
-        <v>1.35</v>
+        <v>1.12</v>
       </c>
       <c r="O5">
-        <v>4.26</v>
+        <v>3.61</v>
       </c>
       <c r="P5">
-        <v>10.6</v>
+        <v>6.1</v>
       </c>
       <c r="Q5">
         <v>0.8</v>
@@ -2436,13 +2436,13 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>9.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Y5">
-        <v>91.7</v>
+        <v>93.2</v>
       </c>
       <c r="Z5">
-        <v>56.3</v>
+        <v>55.9</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2460,25 +2460,25 @@
         <v>156</v>
       </c>
       <c r="AF5">
-        <v>86.7</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="AG5">
-        <v>87.8</v>
+        <v>88.5</v>
       </c>
       <c r="AH5">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AI5">
-        <v>52.6</v>
+        <v>51.6</v>
       </c>
       <c r="AJ5">
-        <v>1009.6</v>
+        <v>1009.7</v>
       </c>
       <c r="AK5">
-        <v>1011.9</v>
+        <v>1012</v>
       </c>
       <c r="AL5">
-        <v>25</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AM5">
         <v>8</v>
@@ -2487,46 +2487,46 @@
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>38.7</v>
+        <v>30</v>
       </c>
       <c r="AP5">
-        <v>592</v>
+        <v>522</v>
       </c>
       <c r="AQ5">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="AR5">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
       <c r="AS5" t="s">
         <v>157</v>
       </c>
       <c r="AT5">
-        <v>322.2</v>
+        <v>325.8</v>
       </c>
       <c r="AU5">
-        <v>-4</v>
+        <v>-4.2</v>
       </c>
       <c r="AV5">
-        <v>-5.9</v>
+        <v>-5.8</v>
       </c>
       <c r="AW5">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
       <c r="AX5">
-        <v>-3.9</v>
+        <v>-4.1</v>
       </c>
       <c r="AY5">
-        <v>-5.2</v>
+        <v>-5.1</v>
       </c>
       <c r="AZ5">
-        <v>-0.7</v>
+        <v>-1</v>
       </c>
       <c r="BA5">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="BB5">
-        <v>-3.5</v>
+        <v>-3.6</v>
       </c>
       <c r="BC5">
         <v>0.5</v>
@@ -2544,13 +2544,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.149</v>
+        <v>1.1486</v>
       </c>
       <c r="BI5" t="s">
         <v>158</v>
       </c>
       <c r="BJ5">
-        <v>1954</v>
+        <v>1972</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2559,34 +2559,34 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>56.9</v>
+        <v>56.3</v>
       </c>
       <c r="BN5">
-        <v>1.017</v>
+        <v>1.015</v>
       </c>
       <c r="BO5">
-        <v>59.4</v>
+        <v>58.7</v>
       </c>
       <c r="BP5">
-        <v>55.3</v>
+        <v>55</v>
       </c>
       <c r="BQ5">
-        <v>53</v>
+        <v>52.8</v>
       </c>
       <c r="BR5">
-        <v>52.9</v>
+        <v>52.8</v>
       </c>
       <c r="BS5">
         <v>55.2</v>
       </c>
       <c r="BT5">
-        <v>10.3</v>
+        <v>9.6</v>
       </c>
       <c r="BU5" t="s">
         <v>69</v>
       </c>
       <c r="BV5">
-        <v>7.5</v>
+        <v>5.7</v>
       </c>
       <c r="BW5" t="s">
         <v>69</v>
@@ -2595,13 +2595,13 @@
         <v>87</v>
       </c>
       <c r="BY5">
-        <v>85.3</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="BZ5">
         <v>5</v>
       </c>
       <c r="CA5">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
     </row>
   </sheetData>
@@ -2703,13 +2703,13 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>89.5</v>
+        <v>87.8</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -2718,7 +2718,7 @@
         <v>4</v>
       </c>
       <c r="J2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="K2">
         <v>-3</v>
@@ -2727,10 +2727,10 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>91.8</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="N2">
-        <v>2327</v>
+        <v>2366</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>